<commit_message>
plots_five_steps_method and flow chart is updated
</commit_message>
<xml_diff>
--- a/data/observation_alpha_beta.xlsx
+++ b/data/observation_alpha_beta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Phd\php_pulsating_heat_pipe\Krp_Analysis\Advanced_PulseHeatPipe_krp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4289ED7D-3208-482C-A879-50DBBA8ED12A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E11E356-21C3-40DC-892E-DF5D3A7FF373}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="final" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">demo!$A$1:$P$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">demo!$A$1:$R$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">final!$A$1:$Q$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
   <si>
     <t>alpha</t>
   </si>
@@ -88,6 +88,12 @@
   <si>
     <t>must repeat</t>
   </si>
+  <si>
+    <t>Change in TR1 [%]</t>
+  </si>
+  <si>
+    <t>Change in TR2 [%]</t>
+  </si>
 </sst>
 </file>
 
@@ -357,7 +363,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -499,6 +505,18 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -781,20 +799,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CC5BB13-84A6-40A9-B2F0-16EBC4A52D5E}">
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="8.54296875" style="3" customWidth="1"/>
     <col min="4" max="8" width="9" style="3" customWidth="1"/>
     <col min="9" max="9" width="8.54296875" style="3" customWidth="1"/>
-    <col min="10" max="11" width="10.26953125" style="3" customWidth="1"/>
-    <col min="12" max="13" width="8.54296875" style="3" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.54296875" style="3" customWidth="1"/>
+    <col min="10" max="13" width="10.26953125" style="3" customWidth="1"/>
+    <col min="14" max="15" width="8.54296875" style="3" customWidth="1"/>
     <col min="16" max="16" width="11.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.54296875" style="3" customWidth="1"/>
+    <col min="18" max="18" width="11.81640625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="5" customFormat="1" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" s="5" customFormat="1" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -826,25 +844,31 @@
         <v>12</v>
       </c>
       <c r="K1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>40</v>
       </c>
@@ -878,27 +902,33 @@
         <f>(D2-G2)/A2</f>
         <v>1.05</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="49">
+        <v>0</v>
+      </c>
+      <c r="L2" s="6">
         <f>(E2-H2)/A2</f>
         <v>0.92500000000000004</v>
       </c>
-      <c r="L2" s="1">
+      <c r="M2" s="49">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
         <v>0.62</v>
       </c>
-      <c r="M2" s="1">
+      <c r="O2" s="1">
         <v>0.75</v>
       </c>
-      <c r="N2" s="1">
+      <c r="P2" s="1">
         <v>-155</v>
       </c>
-      <c r="O2" s="1">
+      <c r="Q2" s="1">
         <v>-190</v>
       </c>
-      <c r="P2" s="1">
+      <c r="R2" s="1">
         <v>-100</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>40</v>
       </c>
@@ -933,26 +963,34 @@
         <v>1.125</v>
       </c>
       <c r="K3" s="6">
-        <f t="shared" ref="K3:K17" si="3">(E3-H3)/A3</f>
+        <f>(J2-J3)/J2</f>
+        <v>-7.1428571428571383E-2</v>
+      </c>
+      <c r="L3" s="6">
+        <f>(E3-H3)/A3</f>
         <v>1.3</v>
       </c>
-      <c r="L3" s="1">
+      <c r="M3" s="6">
+        <f>(L2-L3)/L2</f>
+        <v>-0.40540540540540537</v>
+      </c>
+      <c r="N3" s="1">
         <v>0.7</v>
       </c>
-      <c r="M3" s="1">
+      <c r="O3" s="1">
         <v>0.8</v>
       </c>
-      <c r="N3" s="1">
+      <c r="P3" s="1">
         <v>-140</v>
       </c>
-      <c r="O3" s="1">
+      <c r="Q3" s="1">
         <v>-160</v>
       </c>
-      <c r="P3" s="1">
+      <c r="R3" s="1">
         <v>-0.85</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>40</v>
       </c>
@@ -987,26 +1025,34 @@
         <v>1.125</v>
       </c>
       <c r="K4" s="6">
-        <f t="shared" si="3"/>
+        <f>(J2-J4)/J2</f>
+        <v>-7.1428571428571383E-2</v>
+      </c>
+      <c r="L4" s="6">
+        <f t="shared" ref="L3:L17" si="3">(E4-H4)/A4</f>
         <v>1.3125</v>
       </c>
-      <c r="L4" s="1">
+      <c r="M4" s="6">
+        <f>(L2-L4)/L2</f>
+        <v>-0.41891891891891886</v>
+      </c>
+      <c r="N4" s="1">
         <v>0.7</v>
       </c>
-      <c r="M4" s="1">
+      <c r="O4" s="1">
         <v>0.83</v>
       </c>
-      <c r="N4" s="1">
+      <c r="P4" s="1">
         <v>-130</v>
       </c>
-      <c r="O4" s="1">
+      <c r="Q4" s="1">
         <v>-150</v>
       </c>
-      <c r="P4" s="1">
+      <c r="R4" s="1">
         <v>-90</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>60</v>
       </c>
@@ -1040,27 +1086,29 @@
         <f t="shared" si="2"/>
         <v>0.78333333333333333</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="6"/>
+      <c r="L5" s="6">
         <f t="shared" si="3"/>
         <v>0.6</v>
       </c>
-      <c r="L5" s="1">
+      <c r="M5" s="6"/>
+      <c r="N5" s="1">
         <v>0.65</v>
       </c>
-      <c r="M5" s="1">
-        <v>1</v>
-      </c>
-      <c r="N5" s="1">
+      <c r="O5" s="1">
+        <v>1</v>
+      </c>
+      <c r="P5" s="1">
         <v>-160</v>
       </c>
-      <c r="O5" s="1">
+      <c r="Q5" s="1">
         <v>-180</v>
       </c>
-      <c r="P5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R5" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>60</v>
       </c>
@@ -1094,27 +1142,29 @@
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="6"/>
+      <c r="L6" s="6">
         <f t="shared" si="3"/>
         <v>0.6333333333333333</v>
       </c>
-      <c r="L6" s="1">
+      <c r="M6" s="6"/>
+      <c r="N6" s="1">
         <v>0.75</v>
       </c>
-      <c r="M6" s="1">
-        <v>1</v>
-      </c>
-      <c r="N6" s="1">
+      <c r="O6" s="1">
+        <v>1</v>
+      </c>
+      <c r="P6" s="1">
         <v>-120</v>
       </c>
-      <c r="O6" s="1">
+      <c r="Q6" s="1">
         <v>-150</v>
       </c>
-      <c r="P6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>80</v>
       </c>
@@ -1148,27 +1198,33 @@
         <f t="shared" si="2"/>
         <v>0.6</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="50">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6">
         <f t="shared" si="3"/>
         <v>0.4375</v>
       </c>
-      <c r="L7" s="1">
+      <c r="M7" s="50">
+        <v>0</v>
+      </c>
+      <c r="N7" s="1">
         <v>0.75</v>
       </c>
-      <c r="M7" s="1">
-        <v>1</v>
-      </c>
-      <c r="N7" s="1">
+      <c r="O7" s="1">
+        <v>1</v>
+      </c>
+      <c r="P7" s="1">
         <v>-125</v>
       </c>
-      <c r="O7" s="1">
+      <c r="Q7" s="1">
         <v>-150</v>
       </c>
-      <c r="P7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>80</v>
       </c>
@@ -1203,26 +1259,34 @@
         <v>0.625</v>
       </c>
       <c r="K8" s="6">
+        <f>(J7-J8)/J7</f>
+        <v>-4.1666666666666706E-2</v>
+      </c>
+      <c r="L8" s="6">
         <f t="shared" si="3"/>
         <v>0.5625</v>
       </c>
-      <c r="L8" s="1">
+      <c r="M8" s="6">
+        <f>(L7-L8)/L7</f>
+        <v>-0.2857142857142857</v>
+      </c>
+      <c r="N8" s="1">
         <v>0.8</v>
       </c>
-      <c r="M8" s="1">
-        <v>1</v>
-      </c>
-      <c r="N8" s="1">
+      <c r="O8" s="1">
+        <v>1</v>
+      </c>
+      <c r="P8" s="1">
         <v>-85</v>
       </c>
-      <c r="O8" s="1">
+      <c r="Q8" s="1">
         <v>-100</v>
       </c>
-      <c r="P8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R8" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>80</v>
       </c>
@@ -1257,26 +1321,34 @@
         <v>0.5625</v>
       </c>
       <c r="K9" s="6">
+        <f>(J7-J9)/J7</f>
+        <v>6.2499999999999965E-2</v>
+      </c>
+      <c r="L9" s="6">
         <f t="shared" si="3"/>
         <v>0.45</v>
       </c>
-      <c r="L9" s="1">
+      <c r="M9" s="6">
+        <f>(L7-L9)/L7</f>
+        <v>-2.8571428571428598E-2</v>
+      </c>
+      <c r="N9" s="1">
         <v>0.65</v>
       </c>
-      <c r="M9" s="1">
-        <v>1</v>
-      </c>
-      <c r="N9" s="1">
+      <c r="O9" s="1">
+        <v>1</v>
+      </c>
+      <c r="P9" s="1">
         <v>-160</v>
       </c>
-      <c r="O9" s="1">
+      <c r="Q9" s="1">
         <v>-200</v>
       </c>
-      <c r="P9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>80</v>
       </c>
@@ -1302,35 +1374,43 @@
       <c r="H10" s="2">
         <v>303.5</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="51">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="J10" s="6">
+      <c r="J10" s="52">
         <f t="shared" si="2"/>
         <v>0.71250000000000002</v>
       </c>
-      <c r="K10" s="6">
+      <c r="K10" s="52">
+        <f>(J7-J10)/J7</f>
+        <v>-0.18750000000000008</v>
+      </c>
+      <c r="L10" s="52">
         <f t="shared" si="3"/>
         <v>0.75624999999999998</v>
       </c>
-      <c r="L10" s="2">
+      <c r="M10" s="52">
+        <f>(L7-L10)/L7</f>
+        <v>-0.72857142857142854</v>
+      </c>
+      <c r="N10" s="2">
         <v>0.7</v>
       </c>
-      <c r="M10" s="2">
+      <c r="O10" s="2">
         <v>0.75</v>
       </c>
-      <c r="N10" s="2">
+      <c r="P10" s="2">
         <v>-150</v>
       </c>
-      <c r="O10" s="2">
+      <c r="Q10" s="2">
         <v>-160</v>
       </c>
-      <c r="P10" s="2">
+      <c r="R10" s="2">
         <v>-140</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>100</v>
       </c>
@@ -1365,26 +1445,32 @@
         <v>0.47</v>
       </c>
       <c r="K11" s="6">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6">
         <f t="shared" si="3"/>
         <v>0.4</v>
       </c>
-      <c r="L11" s="1">
+      <c r="M11" s="6">
+        <v>0</v>
+      </c>
+      <c r="N11" s="1">
         <v>0.72</v>
       </c>
-      <c r="M11" s="1">
-        <v>1</v>
-      </c>
-      <c r="N11" s="1">
+      <c r="O11" s="1">
+        <v>1</v>
+      </c>
+      <c r="P11" s="1">
         <v>-130</v>
       </c>
-      <c r="O11" s="1">
+      <c r="Q11" s="1">
         <v>-160</v>
       </c>
-      <c r="P11" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>100</v>
       </c>
@@ -1419,26 +1505,34 @@
         <v>0.47</v>
       </c>
       <c r="K12" s="6">
+        <f>(J11-J12)/J11</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="6">
         <f t="shared" si="3"/>
         <v>0.37</v>
       </c>
-      <c r="L12" s="1">
+      <c r="M12" s="6">
+        <f>(L11-L12)/L11</f>
+        <v>7.5000000000000067E-2</v>
+      </c>
+      <c r="N12" s="1">
         <v>0.75</v>
       </c>
-      <c r="M12" s="1">
-        <v>1</v>
-      </c>
-      <c r="N12" s="1">
+      <c r="O12" s="1">
+        <v>1</v>
+      </c>
+      <c r="P12" s="1">
         <v>-120</v>
       </c>
-      <c r="O12" s="1">
+      <c r="Q12" s="1">
         <v>-130</v>
       </c>
-      <c r="P12" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R12" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>100</v>
       </c>
@@ -1473,26 +1567,34 @@
         <v>0.4</v>
       </c>
       <c r="K13" s="6">
+        <f>(J11-J13)/J11</f>
+        <v>0.14893617021276587</v>
+      </c>
+      <c r="L13" s="6">
         <f t="shared" si="3"/>
         <v>0.32</v>
       </c>
-      <c r="L13" s="1">
+      <c r="M13" s="6">
+        <f>(L11-L13)/L11</f>
+        <v>0.20000000000000004</v>
+      </c>
+      <c r="N13" s="1">
         <v>0.45</v>
       </c>
-      <c r="M13" s="1">
-        <v>1</v>
-      </c>
-      <c r="N13" s="1">
+      <c r="O13" s="1">
+        <v>1</v>
+      </c>
+      <c r="P13" s="1">
         <v>-250</v>
       </c>
-      <c r="O13" s="1">
+      <c r="Q13" s="1">
         <v>-280</v>
       </c>
-      <c r="P13" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>100</v>
       </c>
@@ -1527,26 +1629,34 @@
         <v>0.48</v>
       </c>
       <c r="K14" s="6">
+        <f>(J11-J14)/J11</f>
+        <v>-2.1276595744680871E-2</v>
+      </c>
+      <c r="L14" s="6">
         <f t="shared" si="3"/>
         <v>0.79</v>
       </c>
-      <c r="L14" s="1">
+      <c r="M14" s="6">
+        <f>(L11-L14)/L11</f>
+        <v>-0.97499999999999998</v>
+      </c>
+      <c r="N14" s="1">
         <v>0.67</v>
       </c>
-      <c r="M14" s="1">
+      <c r="O14" s="1">
         <v>0.69</v>
       </c>
-      <c r="N14" s="1">
+      <c r="P14" s="1">
         <v>-270</v>
       </c>
-      <c r="O14" s="1">
+      <c r="Q14" s="1">
         <v>-370</v>
       </c>
-      <c r="P14" s="1">
+      <c r="R14" s="1">
         <v>-240</v>
       </c>
     </row>
-    <row r="15" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>120</v>
       </c>
@@ -1581,26 +1691,32 @@
         <v>0.40833333333333333</v>
       </c>
       <c r="K15" s="6">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6">
         <f t="shared" si="3"/>
         <v>0.34166666666666667</v>
       </c>
-      <c r="L15" s="1">
+      <c r="M15" s="6">
+        <v>0</v>
+      </c>
+      <c r="N15" s="1">
         <v>0.77</v>
       </c>
-      <c r="M15" s="1">
-        <v>1</v>
-      </c>
-      <c r="N15" s="1">
+      <c r="O15" s="1">
+        <v>1</v>
+      </c>
+      <c r="P15" s="1">
         <v>-100</v>
       </c>
-      <c r="O15" s="1">
+      <c r="Q15" s="1">
         <v>-130</v>
       </c>
-      <c r="P15" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R15" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>120</v>
       </c>
@@ -1635,26 +1751,34 @@
         <v>0.38333333333333336</v>
       </c>
       <c r="K16" s="6">
+        <f>(J15-J16)/J15</f>
+        <v>6.122448979591829E-2</v>
+      </c>
+      <c r="L16" s="6">
         <f t="shared" si="3"/>
         <v>0.35833333333333334</v>
       </c>
-      <c r="L16" s="1">
+      <c r="M16" s="6">
+        <f>(L15-L16)/L15</f>
+        <v>-4.8780487804878037E-2</v>
+      </c>
+      <c r="N16" s="1">
         <v>0.8</v>
       </c>
-      <c r="M16" s="1">
-        <v>1</v>
-      </c>
-      <c r="N16" s="1">
+      <c r="O16" s="1">
+        <v>1</v>
+      </c>
+      <c r="P16" s="1">
         <v>-75</v>
       </c>
-      <c r="O16" s="1">
+      <c r="Q16" s="1">
         <v>-85</v>
       </c>
-      <c r="P16" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R16" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>120</v>
       </c>
@@ -1689,26 +1813,34 @@
         <v>0.375</v>
       </c>
       <c r="K17" s="6">
+        <f>(J15-J17)/J15</f>
+        <v>8.1632653061224469E-2</v>
+      </c>
+      <c r="L17" s="6">
         <f t="shared" si="3"/>
         <v>0.29166666666666669</v>
       </c>
-      <c r="L17" s="1">
+      <c r="M17" s="6">
+        <f>(L15-L17)/L15</f>
+        <v>0.14634146341463411</v>
+      </c>
+      <c r="N17" s="1">
         <v>0.6</v>
       </c>
-      <c r="M17" s="1">
-        <v>1</v>
-      </c>
-      <c r="N17" s="1">
+      <c r="O17" s="1">
+        <v>1</v>
+      </c>
+      <c r="P17" s="1">
         <v>-185</v>
       </c>
-      <c r="O17" s="1">
+      <c r="Q17" s="1">
         <v>-230</v>
       </c>
-      <c r="P17" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R17" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="9">
         <v>40</v>
       </c>
@@ -1743,26 +1875,34 @@
         <v>0.9375</v>
       </c>
       <c r="K18" s="6">
+        <f>(J2-J18)/J2</f>
+        <v>0.10714285714285718</v>
+      </c>
+      <c r="L18" s="6">
         <f>(E18-H18)/A18</f>
         <v>1.2375</v>
       </c>
-      <c r="L18" s="1">
+      <c r="M18" s="6">
+        <f>(L2-L18)/L2</f>
+        <v>-0.33783783783783783</v>
+      </c>
+      <c r="N18" s="1">
         <v>0.5</v>
       </c>
-      <c r="M18" s="1">
+      <c r="O18" s="1">
         <v>0.57999999999999996</v>
       </c>
-      <c r="N18" s="1">
+      <c r="P18" s="1">
         <v>-220</v>
       </c>
-      <c r="O18" s="1">
+      <c r="Q18" s="1">
         <v>-235</v>
       </c>
-      <c r="P18" s="1">
+      <c r="R18" s="1">
         <v>-225</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="9">
         <v>40</v>
       </c>
@@ -1797,26 +1937,34 @@
         <v>1.05</v>
       </c>
       <c r="K19" s="6">
+        <f>(J2-J19)/J2</f>
+        <v>0</v>
+      </c>
+      <c r="L19" s="6">
         <f>(E19-H19)/A19</f>
         <v>1.125</v>
       </c>
-      <c r="L19" s="9">
+      <c r="M19" s="6">
+        <f>(L2-L19)/L2</f>
+        <v>-0.21621621621621614</v>
+      </c>
+      <c r="N19" s="9">
         <v>0.6</v>
       </c>
-      <c r="M19" s="9">
+      <c r="O19" s="9">
         <v>0.72</v>
       </c>
-      <c r="N19" s="9">
+      <c r="P19" s="9">
         <v>-175</v>
       </c>
-      <c r="O19" s="9">
+      <c r="Q19" s="9">
         <v>-190</v>
       </c>
-      <c r="P19" s="9">
+      <c r="R19" s="9">
         <v>-120</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="9">
         <v>40</v>
       </c>
@@ -1851,26 +1999,34 @@
         <v>1.125</v>
       </c>
       <c r="K20" s="6">
+        <f>(J2-J20)/J2</f>
+        <v>-7.1428571428571383E-2</v>
+      </c>
+      <c r="L20" s="6">
         <f>(E20-H20)/A20</f>
         <v>1.2</v>
       </c>
-      <c r="L20" s="9">
+      <c r="M20" s="6">
+        <f>(L2-L20)/L2</f>
+        <v>-0.2972972972972972</v>
+      </c>
+      <c r="N20" s="9">
         <v>0.55000000000000004</v>
       </c>
-      <c r="M20" s="9">
+      <c r="O20" s="9">
         <v>0.6</v>
       </c>
-      <c r="N20" s="9">
+      <c r="P20" s="9">
         <v>-230</v>
       </c>
-      <c r="O20" s="9">
+      <c r="Q20" s="9">
         <v>-240</v>
       </c>
-      <c r="P20" s="9">
+      <c r="R20" s="9">
         <v>-220</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="9">
         <v>60</v>
       </c>
@@ -1904,27 +2060,29 @@
         <f t="shared" ref="J21:J31" si="4">(D21-G21)/A21</f>
         <v>0.67500000000000004</v>
       </c>
-      <c r="K21" s="6">
-        <f t="shared" ref="K21:K31" si="5">(E21-H21)/A21</f>
+      <c r="K21" s="6"/>
+      <c r="L21" s="6">
+        <f t="shared" ref="L21:L31" si="5">(E21-H21)/A21</f>
         <v>1.0083333333333333</v>
       </c>
-      <c r="L21" s="1">
+      <c r="M21" s="6"/>
+      <c r="N21" s="1">
         <v>0.62</v>
       </c>
-      <c r="M21" s="1">
+      <c r="O21" s="1">
         <v>0.8</v>
       </c>
-      <c r="N21" s="1">
+      <c r="P21" s="1">
         <v>-155</v>
       </c>
-      <c r="O21" s="1">
+      <c r="Q21" s="1">
         <v>-175</v>
       </c>
-      <c r="P21" s="1">
+      <c r="R21" s="1">
         <v>-90</v>
       </c>
     </row>
-    <row r="22" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="9">
         <v>60</v>
       </c>
@@ -1958,27 +2116,29 @@
         <f>(D22-G22)/A22</f>
         <v>0.6166666666666667</v>
       </c>
-      <c r="K22" s="6">
+      <c r="K22" s="6"/>
+      <c r="L22" s="6">
         <f>(E22-H22)/A22</f>
         <v>0.51666666666666672</v>
       </c>
-      <c r="L22" s="9">
+      <c r="M22" s="6"/>
+      <c r="N22" s="9">
         <v>0.5</v>
       </c>
-      <c r="M22" s="9">
+      <c r="O22" s="9">
         <v>0.74</v>
       </c>
-      <c r="N22" s="9">
+      <c r="P22" s="9">
         <v>-220</v>
       </c>
-      <c r="O22" s="9">
+      <c r="Q22" s="9">
         <v>-225</v>
       </c>
-      <c r="P22" s="9">
+      <c r="R22" s="9">
         <v>-75</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="9">
         <v>60</v>
       </c>
@@ -2012,27 +2172,29 @@
         <f>(D23-G23)/A23</f>
         <v>0.73333333333333328</v>
       </c>
-      <c r="K23" s="6">
+      <c r="K23" s="6"/>
+      <c r="L23" s="6">
         <f>(E23-H23)/A23</f>
         <v>0.58333333333333337</v>
       </c>
-      <c r="L23" s="9">
+      <c r="M23" s="6"/>
+      <c r="N23" s="9">
         <v>0.68</v>
       </c>
-      <c r="M23" s="9">
+      <c r="O23" s="9">
         <v>0.78</v>
       </c>
-      <c r="N23" s="9">
+      <c r="P23" s="9">
         <v>-130</v>
       </c>
-      <c r="O23" s="9">
+      <c r="Q23" s="9">
         <v>-260</v>
       </c>
-      <c r="P23" s="9">
+      <c r="R23" s="9">
         <v>-70</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="9">
         <v>80</v>
       </c>
@@ -2067,26 +2229,34 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="K24" s="6">
+        <f>(J7-J24)/J7</f>
+        <v>8.3333333333333232E-2</v>
+      </c>
+      <c r="L24" s="6">
         <f>(E24-H24)/A24</f>
         <v>0.38750000000000001</v>
       </c>
-      <c r="L24" s="9">
+      <c r="M24" s="6">
+        <f>(L7-L24)/L7</f>
+        <v>0.11428571428571425</v>
+      </c>
+      <c r="N24" s="9">
         <v>0.62</v>
       </c>
-      <c r="M24" s="9">
-        <v>1</v>
-      </c>
-      <c r="N24" s="9">
+      <c r="O24" s="9">
+        <v>1</v>
+      </c>
+      <c r="P24" s="9">
         <v>-160</v>
       </c>
-      <c r="O24" s="9">
+      <c r="Q24" s="9">
         <v>-230</v>
       </c>
-      <c r="P24" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R24" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="9">
         <v>80</v>
       </c>
@@ -2121,26 +2291,34 @@
         <v>0.52500000000000002</v>
       </c>
       <c r="K25" s="6">
+        <f>(J7-J25)/J7</f>
+        <v>0.12499999999999993</v>
+      </c>
+      <c r="L25" s="6">
         <f>(E25-H25)/A25</f>
         <v>0.35</v>
       </c>
-      <c r="L25" s="9">
+      <c r="M25" s="6">
+        <f>(L7-L25)/L7</f>
+        <v>0.20000000000000004</v>
+      </c>
+      <c r="N25" s="9">
         <v>0.46</v>
       </c>
-      <c r="M25" s="9">
+      <c r="O25" s="9">
         <v>0.92</v>
       </c>
-      <c r="N25" s="9">
+      <c r="P25" s="9">
         <v>-255</v>
       </c>
-      <c r="O25" s="9">
+      <c r="Q25" s="9">
         <v>-300</v>
       </c>
-      <c r="P25" s="9">
+      <c r="R25" s="9">
         <v>-20</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="9">
         <v>100</v>
       </c>
@@ -2175,26 +2353,34 @@
         <v>0.46</v>
       </c>
       <c r="K26" s="6">
+        <f>(J11-J26)/J11</f>
+        <v>2.1276595744680753E-2</v>
+      </c>
+      <c r="L26" s="6">
         <f t="shared" si="5"/>
         <v>0.66</v>
       </c>
-      <c r="L26" s="1">
+      <c r="M26" s="6">
+        <f>(L11-L26)/L11</f>
+        <v>-0.65</v>
+      </c>
+      <c r="N26" s="1">
         <v>0.55000000000000004</v>
       </c>
-      <c r="M26" s="1">
-        <v>1</v>
-      </c>
-      <c r="N26" s="1">
+      <c r="O26" s="1">
+        <v>1</v>
+      </c>
+      <c r="P26" s="1">
         <v>-150</v>
       </c>
-      <c r="O26" s="1">
+      <c r="Q26" s="1">
         <v>-170</v>
       </c>
-      <c r="P26" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R26" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="9">
         <v>100</v>
       </c>
@@ -2229,26 +2415,34 @@
         <v>0.39</v>
       </c>
       <c r="K27" s="6">
+        <f>(J11-J27)/J11</f>
+        <v>0.17021276595744672</v>
+      </c>
+      <c r="L27" s="6">
         <f>(E27-H27)/A27</f>
         <v>0.27</v>
       </c>
-      <c r="L27" s="9">
+      <c r="M27" s="6">
+        <f>(L11-L27)/L11</f>
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="N27" s="9">
         <v>0.48</v>
       </c>
-      <c r="M27" s="9">
-        <v>1</v>
-      </c>
-      <c r="N27" s="9">
+      <c r="O27" s="9">
+        <v>1</v>
+      </c>
+      <c r="P27" s="9">
         <v>-220</v>
       </c>
-      <c r="O27" s="9">
+      <c r="Q27" s="9">
         <v>-250</v>
       </c>
-      <c r="P27" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R27" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="9">
         <v>100</v>
       </c>
@@ -2283,26 +2477,34 @@
         <v>0.4</v>
       </c>
       <c r="K28" s="6">
+        <f>(J11-J28)/J11</f>
+        <v>0.14893617021276587</v>
+      </c>
+      <c r="L28" s="6">
         <f>(E28-H28)/A28</f>
         <v>0.26</v>
       </c>
-      <c r="L28" s="9">
+      <c r="M28" s="6">
+        <f>(L11-L28)/L11</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="N28" s="9">
         <v>0.6</v>
       </c>
-      <c r="M28" s="9">
-        <v>1</v>
-      </c>
-      <c r="N28" s="9">
+      <c r="O28" s="9">
+        <v>1</v>
+      </c>
+      <c r="P28" s="9">
         <v>-150</v>
       </c>
-      <c r="O28" s="9">
+      <c r="Q28" s="9">
         <v>-210</v>
       </c>
-      <c r="P28" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R28" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="9">
         <v>120</v>
       </c>
@@ -2337,26 +2539,34 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="K29" s="6">
+        <f>(J15-J29)/J15</f>
+        <v>-2.0408163265306187E-2</v>
+      </c>
+      <c r="L29" s="6">
         <f t="shared" si="5"/>
         <v>0.46666666666666667</v>
       </c>
-      <c r="L29" s="1">
+      <c r="M29" s="6">
+        <f>(L15-L29)/L15</f>
+        <v>-0.36585365853658536</v>
+      </c>
+      <c r="N29" s="1">
         <v>0.6</v>
       </c>
-      <c r="M29" s="1">
-        <v>1</v>
-      </c>
-      <c r="N29" s="1">
+      <c r="O29" s="1">
+        <v>1</v>
+      </c>
+      <c r="P29" s="1">
         <v>215</v>
       </c>
-      <c r="O29" s="1">
+      <c r="Q29" s="1">
         <v>-230</v>
       </c>
-      <c r="P29" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R29" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="9">
         <v>120</v>
       </c>
@@ -2391,26 +2601,34 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="K30" s="6">
+        <f>(J15-J30)/J15</f>
+        <v>0.18367346938775514</v>
+      </c>
+      <c r="L30" s="6">
         <f t="shared" si="5"/>
         <v>0.20833333333333334</v>
       </c>
-      <c r="L30" s="9">
+      <c r="M30" s="6">
+        <f>(L15-L30)/L15</f>
+        <v>0.3902439024390244</v>
+      </c>
+      <c r="N30" s="9">
         <v>0.54</v>
       </c>
-      <c r="M30" s="9">
-        <v>1</v>
-      </c>
-      <c r="N30" s="9">
+      <c r="O30" s="9">
+        <v>1</v>
+      </c>
+      <c r="P30" s="9">
         <v>-215</v>
       </c>
-      <c r="O30" s="9">
+      <c r="Q30" s="9">
         <v>-230</v>
       </c>
-      <c r="P30" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="R30" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="20" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="9">
         <v>120</v>
       </c>
@@ -2445,22 +2663,30 @@
         <v>0.32500000000000001</v>
       </c>
       <c r="K31" s="6">
+        <f>(J15-J31)/J15</f>
+        <v>0.20408163265306117</v>
+      </c>
+      <c r="L31" s="6">
         <f t="shared" si="5"/>
         <v>0.23333333333333334</v>
       </c>
-      <c r="L31" s="9">
+      <c r="M31" s="6">
+        <f>(L15-L31)/L15</f>
+        <v>0.31707317073170732</v>
+      </c>
+      <c r="N31" s="9">
         <v>0.52</v>
       </c>
-      <c r="M31" s="9">
-        <v>1</v>
-      </c>
-      <c r="N31" s="9">
+      <c r="O31" s="9">
+        <v>1</v>
+      </c>
+      <c r="P31" s="9">
         <v>-200</v>
       </c>
-      <c r="O31" s="9">
+      <c r="Q31" s="9">
         <v>-250</v>
       </c>
-      <c r="P31" s="9">
+      <c r="R31" s="9">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
plots_five_steps_method is updated For 60W, (90,0) may be leakage. Remove- %change TR
</commit_message>
<xml_diff>
--- a/data/observation_alpha_beta.xlsx
+++ b/data/observation_alpha_beta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Phd\php_pulsating_heat_pipe\Krp_Analysis\Advanced_PulseHeatPipe_krp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE050A59-0AA2-43C9-9235-D380B1992CA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC9E0F1-BBD3-4453-A86D-081082238606}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="60" windowWidth="18200" windowHeight="8510" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1234,19 +1234,13 @@
         <v>0.78333333333333333</v>
       </c>
       <c r="K5" s="54"/>
-      <c r="L5" s="55">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="L5" s="55"/>
       <c r="M5" s="54">
         <f t="shared" ref="M5:M17" si="5">(E6-H6)/A6</f>
         <v>0.6333333333333333</v>
       </c>
       <c r="N5" s="54"/>
-      <c r="O5" s="55">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="O5" s="55"/>
       <c r="P5" s="55">
         <v>0.65</v>
       </c>
@@ -1298,19 +1292,13 @@
         <v>0.75</v>
       </c>
       <c r="K6" s="54"/>
-      <c r="L6" s="55">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="L6" s="55"/>
       <c r="M6" s="54">
         <f t="shared" si="5"/>
         <v>0.4375</v>
       </c>
       <c r="N6" s="54"/>
-      <c r="O6" s="55">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="O6" s="55"/>
       <c r="P6" s="55">
         <v>0.75</v>
       </c>
@@ -2330,19 +2318,13 @@
         <v>0.67500000000000004</v>
       </c>
       <c r="K21" s="54"/>
-      <c r="L21" s="55">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="L21" s="55"/>
       <c r="M21" s="54">
         <f t="shared" si="6"/>
         <v>1.0083333333333333</v>
       </c>
       <c r="N21" s="54"/>
-      <c r="O21" s="55">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="O21" s="55"/>
       <c r="P21" s="55">
         <v>0.62</v>
       </c>
@@ -2394,19 +2376,13 @@
         <v>0.6166666666666667</v>
       </c>
       <c r="K22" s="54"/>
-      <c r="L22" s="55">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="L22" s="55"/>
       <c r="M22" s="54">
         <f t="shared" si="6"/>
         <v>0.51666666666666672</v>
       </c>
       <c r="N22" s="54"/>
-      <c r="O22" s="55">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="O22" s="55"/>
       <c r="P22" s="55">
         <v>0.5</v>
       </c>
@@ -2458,19 +2434,13 @@
         <v>0.73333333333333328</v>
       </c>
       <c r="K23" s="54"/>
-      <c r="L23" s="55">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
+      <c r="L23" s="55"/>
       <c r="M23" s="54">
         <f t="shared" si="6"/>
         <v>0.58333333333333337</v>
       </c>
       <c r="N23" s="54"/>
-      <c r="O23" s="55">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
+      <c r="O23" s="55"/>
       <c r="P23" s="55">
         <v>0.68</v>
       </c>

</xml_diff>

<commit_message>
meta_table_data_5_5 is updated for JTACC_Hungary
</commit_message>
<xml_diff>
--- a/data/observation_alpha_beta.xlsx
+++ b/data/observation_alpha_beta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Phd\php_pulsating_heat_pipe\Krp_Analysis\Advanced_PulseHeatPipe_krp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC9E0F1-BBD3-4453-A86D-081082238606}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBBCA33-E16F-472A-A796-78673E6338E9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="60" windowWidth="18200" windowHeight="8510" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -103,7 +103,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,6 +122,13 @@
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -427,7 +434,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -507,15 +514,9 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -525,9 +526,6 @@
     <xf numFmtId="4" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="4" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -566,9 +564,6 @@
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -607,6 +602,34 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -915,20 +938,20 @@
   <dimension ref="A1:T31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="8.54296875" style="49" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="9" style="49" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.54296875" style="49" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.26953125" style="50" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.453125" style="50" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.453125" style="50" customWidth="1"/>
-    <col min="13" max="13" width="10.26953125" style="50" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.26953125" style="50" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.26953125" style="50" customWidth="1"/>
-    <col min="16" max="16" width="8.54296875" style="51" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.54296875" style="49" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.81640625" style="49" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.54296875" style="49" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.81640625" style="49" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="8.54296875" style="45" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="9" style="45" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.54296875" style="45" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.26953125" style="46" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.453125" style="46" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.453125" style="46" customWidth="1"/>
+    <col min="13" max="13" width="10.26953125" style="46" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.26953125" style="46" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.26953125" style="46" customWidth="1"/>
+    <col min="16" max="16" width="8.54296875" style="47" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.54296875" style="45" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.81640625" style="45" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.54296875" style="45" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.81640625" style="45" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -994,2026 +1017,2026 @@
       </c>
     </row>
     <row r="2" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="53">
+      <c r="A2" s="49">
         <v>40</v>
       </c>
-      <c r="B2" s="53">
+      <c r="B2" s="49">
         <v>90</v>
       </c>
-      <c r="C2" s="53">
-        <v>0</v>
-      </c>
-      <c r="D2" s="53">
+      <c r="C2" s="49">
+        <v>0</v>
+      </c>
+      <c r="D2" s="49">
         <v>348</v>
       </c>
-      <c r="E2" s="53">
+      <c r="E2" s="49">
         <v>352</v>
       </c>
-      <c r="F2" s="53">
+      <c r="F2" s="49">
         <f t="shared" ref="F2:F31" si="0">(E2-D2)</f>
         <v>4</v>
       </c>
-      <c r="G2" s="53">
+      <c r="G2" s="49">
         <v>306</v>
       </c>
-      <c r="H2" s="53">
+      <c r="H2" s="49">
         <v>315</v>
       </c>
-      <c r="I2" s="53">
+      <c r="I2" s="49">
         <f t="shared" ref="I2:I31" si="1">(H2-G2)</f>
         <v>9</v>
       </c>
-      <c r="J2" s="54">
+      <c r="J2" s="50">
         <f t="shared" ref="J2:J31" si="2">(D2-G2)/A2</f>
         <v>1.05</v>
       </c>
-      <c r="K2" s="55">
-        <v>0</v>
-      </c>
-      <c r="L2" s="55">
-        <v>0</v>
-      </c>
-      <c r="M2" s="54">
+      <c r="K2" s="51">
+        <v>0</v>
+      </c>
+      <c r="L2" s="51">
+        <v>0</v>
+      </c>
+      <c r="M2" s="50">
         <f>(E2-H2)/A2</f>
         <v>0.92500000000000004</v>
       </c>
-      <c r="N2" s="55">
-        <v>0</v>
-      </c>
-      <c r="O2" s="55">
-        <v>0</v>
-      </c>
-      <c r="P2" s="55">
+      <c r="N2" s="51">
+        <v>0</v>
+      </c>
+      <c r="O2" s="51">
+        <v>0</v>
+      </c>
+      <c r="P2" s="51">
         <v>0.62</v>
       </c>
-      <c r="Q2" s="55">
+      <c r="Q2" s="51">
         <v>0.75</v>
       </c>
-      <c r="R2" s="53">
+      <c r="R2" s="49">
         <v>-155</v>
       </c>
-      <c r="S2" s="53">
+      <c r="S2" s="49">
         <v>-190</v>
       </c>
-      <c r="T2" s="53">
+      <c r="T2" s="49">
         <v>-100</v>
       </c>
     </row>
     <row r="3" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="53">
+      <c r="A3" s="49">
         <v>40</v>
       </c>
-      <c r="B3" s="53">
+      <c r="B3" s="49">
         <v>60</v>
       </c>
-      <c r="C3" s="53">
-        <v>0</v>
-      </c>
-      <c r="D3" s="53">
+      <c r="C3" s="49">
+        <v>0</v>
+      </c>
+      <c r="D3" s="49">
         <v>349</v>
       </c>
-      <c r="E3" s="53">
+      <c r="E3" s="49">
         <v>357</v>
       </c>
-      <c r="F3" s="53">
+      <c r="F3" s="49">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="G3" s="53">
+      <c r="G3" s="49">
         <v>304</v>
       </c>
-      <c r="H3" s="53">
+      <c r="H3" s="49">
         <v>305</v>
       </c>
-      <c r="I3" s="56">
+      <c r="I3" s="52">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J3" s="54">
+      <c r="J3" s="50">
         <f t="shared" si="2"/>
         <v>1.125</v>
       </c>
-      <c r="K3" s="54">
+      <c r="K3" s="50">
         <f>(J2-J3)/J2</f>
         <v>-7.1428571428571383E-2</v>
       </c>
-      <c r="L3" s="55">
+      <c r="L3" s="51">
         <f t="shared" ref="L3:L31" si="3">K3*100</f>
         <v>-7.1428571428571379</v>
       </c>
-      <c r="M3" s="54">
+      <c r="M3" s="50">
         <f>(E3-H3)/A3</f>
         <v>1.3</v>
       </c>
-      <c r="N3" s="54">
+      <c r="N3" s="50">
         <f>(M2-M3)/M2</f>
         <v>-0.40540540540540537</v>
       </c>
-      <c r="O3" s="55">
+      <c r="O3" s="51">
         <f t="shared" ref="O3:O31" si="4">N3*100</f>
         <v>-40.54054054054054</v>
       </c>
-      <c r="P3" s="55">
+      <c r="P3" s="51">
         <v>0.7</v>
       </c>
-      <c r="Q3" s="55">
+      <c r="Q3" s="51">
         <v>0.8</v>
       </c>
-      <c r="R3" s="53">
+      <c r="R3" s="49">
         <v>-140</v>
       </c>
-      <c r="S3" s="53">
+      <c r="S3" s="49">
         <v>-160</v>
       </c>
-      <c r="T3" s="55">
+      <c r="T3" s="51">
         <v>-0.85</v>
       </c>
     </row>
     <row r="4" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="53">
+      <c r="A4" s="49">
         <v>40</v>
       </c>
-      <c r="B4" s="53">
+      <c r="B4" s="49">
         <v>30</v>
       </c>
-      <c r="C4" s="53">
-        <v>0</v>
-      </c>
-      <c r="D4" s="53">
+      <c r="C4" s="49">
+        <v>0</v>
+      </c>
+      <c r="D4" s="49">
         <v>349</v>
       </c>
-      <c r="E4" s="55">
+      <c r="E4" s="51">
         <v>358.5</v>
       </c>
-      <c r="F4" s="55">
+      <c r="F4" s="51">
         <f t="shared" si="0"/>
         <v>9.5</v>
       </c>
-      <c r="G4" s="53">
+      <c r="G4" s="49">
         <v>304</v>
       </c>
-      <c r="H4" s="53">
+      <c r="H4" s="49">
         <v>306</v>
       </c>
-      <c r="I4" s="56">
+      <c r="I4" s="52">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="J4" s="54">
+      <c r="J4" s="50">
         <f t="shared" si="2"/>
         <v>1.125</v>
       </c>
-      <c r="K4" s="54">
+      <c r="K4" s="50">
         <f>(J2-J4)/J2</f>
         <v>-7.1428571428571383E-2</v>
       </c>
-      <c r="L4" s="55">
+      <c r="L4" s="51">
         <f t="shared" si="3"/>
         <v>-7.1428571428571379</v>
       </c>
-      <c r="M4" s="54">
+      <c r="M4" s="50">
         <f>(E4-H4)/A4</f>
         <v>1.3125</v>
       </c>
-      <c r="N4" s="54">
+      <c r="N4" s="50">
         <f>(M2-M4)/M2</f>
         <v>-0.41891891891891886</v>
       </c>
-      <c r="O4" s="55">
+      <c r="O4" s="51">
         <f t="shared" si="4"/>
         <v>-41.891891891891888</v>
       </c>
-      <c r="P4" s="55">
+      <c r="P4" s="51">
         <v>0.7</v>
       </c>
-      <c r="Q4" s="55">
+      <c r="Q4" s="51">
         <v>0.83</v>
       </c>
-      <c r="R4" s="53">
+      <c r="R4" s="49">
         <v>-130</v>
       </c>
-      <c r="S4" s="53">
+      <c r="S4" s="49">
         <v>-150</v>
       </c>
-      <c r="T4" s="53">
+      <c r="T4" s="49">
         <v>-90</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="53">
+      <c r="A5" s="49">
         <v>60</v>
       </c>
-      <c r="B5" s="53">
+      <c r="B5" s="49">
         <v>60</v>
       </c>
-      <c r="C5" s="53">
-        <v>0</v>
-      </c>
-      <c r="D5" s="53">
+      <c r="C5" s="49">
+        <v>0</v>
+      </c>
+      <c r="D5" s="49">
         <v>350</v>
       </c>
-      <c r="E5" s="53">
+      <c r="E5" s="49">
         <v>355</v>
       </c>
-      <c r="F5" s="53">
+      <c r="F5" s="49">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="G5" s="53">
+      <c r="G5" s="49">
         <v>303</v>
       </c>
-      <c r="H5" s="53">
+      <c r="H5" s="49">
         <v>319</v>
       </c>
-      <c r="I5" s="56">
+      <c r="I5" s="52">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="J5" s="54">
+      <c r="J5" s="50">
         <f t="shared" si="2"/>
         <v>0.78333333333333333</v>
       </c>
-      <c r="K5" s="54"/>
-      <c r="L5" s="55"/>
-      <c r="M5" s="54">
+      <c r="K5" s="50"/>
+      <c r="L5" s="51"/>
+      <c r="M5" s="50">
         <f t="shared" ref="M5:M17" si="5">(E6-H6)/A6</f>
         <v>0.6333333333333333</v>
       </c>
-      <c r="N5" s="54"/>
-      <c r="O5" s="55"/>
-      <c r="P5" s="55">
+      <c r="N5" s="50"/>
+      <c r="O5" s="51"/>
+      <c r="P5" s="51">
         <v>0.65</v>
       </c>
-      <c r="Q5" s="53">
+      <c r="Q5" s="49">
         <v>1</v>
       </c>
-      <c r="R5" s="53">
+      <c r="R5" s="49">
         <v>-160</v>
       </c>
-      <c r="S5" s="53">
+      <c r="S5" s="49">
         <v>-180</v>
       </c>
-      <c r="T5" s="53">
+      <c r="T5" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="53">
+      <c r="A6" s="49">
         <v>60</v>
       </c>
-      <c r="B6" s="53">
+      <c r="B6" s="49">
         <v>30</v>
       </c>
-      <c r="C6" s="53">
-        <v>0</v>
-      </c>
-      <c r="D6" s="53">
+      <c r="C6" s="49">
+        <v>0</v>
+      </c>
+      <c r="D6" s="49">
         <v>350</v>
       </c>
-      <c r="E6" s="53">
+      <c r="E6" s="49">
         <v>359</v>
       </c>
-      <c r="F6" s="53">
+      <c r="F6" s="49">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="G6" s="53">
+      <c r="G6" s="49">
         <v>305</v>
       </c>
-      <c r="H6" s="53">
+      <c r="H6" s="49">
         <v>321</v>
       </c>
-      <c r="I6" s="56">
+      <c r="I6" s="52">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="J6" s="54">
+      <c r="J6" s="50">
         <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
-      <c r="K6" s="54"/>
-      <c r="L6" s="55"/>
-      <c r="M6" s="54">
+      <c r="K6" s="50"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="50">
         <f t="shared" si="5"/>
         <v>0.4375</v>
       </c>
-      <c r="N6" s="54"/>
-      <c r="O6" s="55"/>
-      <c r="P6" s="55">
+      <c r="N6" s="50"/>
+      <c r="O6" s="51"/>
+      <c r="P6" s="51">
         <v>0.75</v>
       </c>
-      <c r="Q6" s="53">
+      <c r="Q6" s="49">
         <v>1</v>
       </c>
-      <c r="R6" s="53">
+      <c r="R6" s="49">
         <v>-120</v>
       </c>
-      <c r="S6" s="53">
+      <c r="S6" s="49">
         <v>-150</v>
       </c>
-      <c r="T6" s="53">
+      <c r="T6" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="53">
+      <c r="A7" s="49">
         <v>80</v>
       </c>
-      <c r="B7" s="53">
+      <c r="B7" s="49">
         <v>90</v>
       </c>
-      <c r="C7" s="53">
-        <v>0</v>
-      </c>
-      <c r="D7" s="53">
+      <c r="C7" s="49">
+        <v>0</v>
+      </c>
+      <c r="D7" s="49">
         <v>350</v>
       </c>
-      <c r="E7" s="53">
+      <c r="E7" s="49">
         <v>355</v>
       </c>
-      <c r="F7" s="53">
+      <c r="F7" s="49">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="G7" s="53">
+      <c r="G7" s="49">
         <v>302</v>
       </c>
-      <c r="H7" s="53">
+      <c r="H7" s="49">
         <v>320</v>
       </c>
-      <c r="I7" s="56">
+      <c r="I7" s="52">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="J7" s="54">
+      <c r="J7" s="50">
         <f t="shared" si="2"/>
         <v>0.6</v>
       </c>
-      <c r="K7" s="55">
-        <v>0</v>
-      </c>
-      <c r="L7" s="55">
-        <v>0</v>
-      </c>
-      <c r="M7" s="54">
+      <c r="K7" s="51">
+        <v>0</v>
+      </c>
+      <c r="L7" s="51">
+        <v>0</v>
+      </c>
+      <c r="M7" s="50">
         <f t="shared" si="5"/>
         <v>0.5625</v>
       </c>
-      <c r="N7" s="55">
-        <v>0</v>
-      </c>
-      <c r="O7" s="55">
-        <v>0</v>
-      </c>
-      <c r="P7" s="55">
+      <c r="N7" s="51">
+        <v>0</v>
+      </c>
+      <c r="O7" s="51">
+        <v>0</v>
+      </c>
+      <c r="P7" s="51">
         <v>0.75</v>
       </c>
-      <c r="Q7" s="53">
+      <c r="Q7" s="49">
         <v>1</v>
       </c>
-      <c r="R7" s="53">
+      <c r="R7" s="49">
         <v>-125</v>
       </c>
-      <c r="S7" s="53">
+      <c r="S7" s="49">
         <v>-150</v>
       </c>
-      <c r="T7" s="53">
+      <c r="T7" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="53">
+      <c r="A8" s="49">
         <v>80</v>
       </c>
-      <c r="B8" s="53">
+      <c r="B8" s="49">
         <v>60</v>
       </c>
-      <c r="C8" s="53">
-        <v>0</v>
-      </c>
-      <c r="D8" s="53">
+      <c r="C8" s="49">
+        <v>0</v>
+      </c>
+      <c r="D8" s="49">
         <v>355</v>
       </c>
-      <c r="E8" s="53">
+      <c r="E8" s="49">
         <v>358</v>
       </c>
-      <c r="F8" s="53">
+      <c r="F8" s="49">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G8" s="53">
+      <c r="G8" s="49">
         <v>305</v>
       </c>
-      <c r="H8" s="53">
+      <c r="H8" s="49">
         <v>313</v>
       </c>
-      <c r="I8" s="56">
+      <c r="I8" s="52">
         <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="J8" s="54">
+      <c r="J8" s="50">
         <f t="shared" si="2"/>
         <v>0.625</v>
       </c>
-      <c r="K8" s="54">
+      <c r="K8" s="50">
         <f>(J7-J8)/J7</f>
         <v>-4.1666666666666706E-2</v>
       </c>
-      <c r="L8" s="55">
+      <c r="L8" s="51">
         <f t="shared" si="3"/>
         <v>-4.1666666666666705</v>
       </c>
-      <c r="M8" s="54">
+      <c r="M8" s="50">
         <f t="shared" si="5"/>
         <v>0.45</v>
       </c>
-      <c r="N8" s="54">
+      <c r="N8" s="50">
         <f>(M7-M8)/M7</f>
         <v>0.19999999999999998</v>
       </c>
-      <c r="O8" s="55">
+      <c r="O8" s="51">
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="P8" s="55">
+      <c r="P8" s="51">
         <v>0.8</v>
       </c>
-      <c r="Q8" s="53">
+      <c r="Q8" s="49">
         <v>1</v>
       </c>
-      <c r="R8" s="53">
+      <c r="R8" s="49">
         <v>-85</v>
       </c>
-      <c r="S8" s="53">
+      <c r="S8" s="49">
         <v>-100</v>
       </c>
-      <c r="T8" s="53">
+      <c r="T8" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="53">
+      <c r="A9" s="49">
         <v>80</v>
       </c>
-      <c r="B9" s="53">
+      <c r="B9" s="49">
         <v>30</v>
       </c>
-      <c r="C9" s="53">
-        <v>0</v>
-      </c>
-      <c r="D9" s="53">
+      <c r="C9" s="49">
+        <v>0</v>
+      </c>
+      <c r="D9" s="49">
         <v>348</v>
       </c>
-      <c r="E9" s="53">
+      <c r="E9" s="49">
         <v>358</v>
       </c>
-      <c r="F9" s="53">
+      <c r="F9" s="49">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="G9" s="53">
+      <c r="G9" s="49">
         <v>303</v>
       </c>
-      <c r="H9" s="53">
+      <c r="H9" s="49">
         <v>322</v>
       </c>
-      <c r="I9" s="56">
+      <c r="I9" s="52">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
-      <c r="J9" s="54">
+      <c r="J9" s="50">
         <f t="shared" si="2"/>
         <v>0.5625</v>
       </c>
-      <c r="K9" s="54">
+      <c r="K9" s="50">
         <f>(J7-J9)/J7</f>
         <v>6.2499999999999965E-2</v>
       </c>
-      <c r="L9" s="55">
+      <c r="L9" s="51">
         <f t="shared" si="3"/>
         <v>6.2499999999999964</v>
       </c>
-      <c r="M9" s="54">
+      <c r="M9" s="50">
         <f t="shared" si="5"/>
         <v>0.75624999999999998</v>
       </c>
-      <c r="N9" s="54">
+      <c r="N9" s="50">
         <f>(M7-M9)/M7</f>
         <v>-0.34444444444444439</v>
       </c>
-      <c r="O9" s="55">
+      <c r="O9" s="51">
         <f t="shared" si="4"/>
         <v>-34.444444444444436</v>
       </c>
-      <c r="P9" s="55">
+      <c r="P9" s="51">
         <v>0.65</v>
       </c>
-      <c r="Q9" s="53">
+      <c r="Q9" s="49">
         <v>1</v>
       </c>
-      <c r="R9" s="53">
+      <c r="R9" s="49">
         <v>-160</v>
       </c>
-      <c r="S9" s="53">
+      <c r="S9" s="49">
         <v>-200</v>
       </c>
-      <c r="T9" s="53">
+      <c r="T9" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:20" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="57">
+      <c r="A10" s="53">
         <v>80</v>
       </c>
-      <c r="B10" s="57">
-        <v>0</v>
-      </c>
-      <c r="C10" s="57">
-        <v>0</v>
-      </c>
-      <c r="D10" s="57">
+      <c r="B10" s="53">
+        <v>0</v>
+      </c>
+      <c r="C10" s="53">
+        <v>0</v>
+      </c>
+      <c r="D10" s="53">
         <v>360</v>
       </c>
-      <c r="E10" s="57">
+      <c r="E10" s="53">
         <v>364</v>
       </c>
-      <c r="F10" s="57">
+      <c r="F10" s="53">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G10" s="57">
+      <c r="G10" s="53">
         <v>303</v>
       </c>
-      <c r="H10" s="58">
+      <c r="H10" s="54">
         <v>303.5</v>
       </c>
-      <c r="I10" s="59">
+      <c r="I10" s="55">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="J10" s="60">
+      <c r="J10" s="56">
         <f t="shared" si="2"/>
         <v>0.71250000000000002</v>
       </c>
-      <c r="K10" s="60">
+      <c r="K10" s="56">
         <f>(J7-J10)/J7</f>
         <v>-0.18750000000000008</v>
       </c>
-      <c r="L10" s="55">
+      <c r="L10" s="51">
         <f t="shared" si="3"/>
         <v>-18.750000000000007</v>
       </c>
-      <c r="M10" s="60">
+      <c r="M10" s="56">
         <f t="shared" si="5"/>
         <v>0.4</v>
       </c>
-      <c r="N10" s="60">
+      <c r="N10" s="56">
         <f>(M7-M10)/M7</f>
         <v>0.28888888888888886</v>
       </c>
-      <c r="O10" s="55">
+      <c r="O10" s="51">
         <f t="shared" si="4"/>
         <v>28.888888888888886</v>
       </c>
-      <c r="P10" s="58">
+      <c r="P10" s="54">
         <v>0.7</v>
       </c>
-      <c r="Q10" s="58">
+      <c r="Q10" s="54">
         <v>0.75</v>
       </c>
-      <c r="R10" s="57">
+      <c r="R10" s="53">
         <v>-150</v>
       </c>
-      <c r="S10" s="57">
+      <c r="S10" s="53">
         <v>-160</v>
       </c>
-      <c r="T10" s="57">
+      <c r="T10" s="53">
         <v>-140</v>
       </c>
     </row>
     <row r="11" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="53">
+      <c r="A11" s="49">
         <v>100</v>
       </c>
-      <c r="B11" s="53">
+      <c r="B11" s="49">
         <v>90</v>
       </c>
-      <c r="C11" s="53">
-        <v>0</v>
-      </c>
-      <c r="D11" s="53">
+      <c r="C11" s="49">
+        <v>0</v>
+      </c>
+      <c r="D11" s="49">
         <v>352</v>
       </c>
-      <c r="E11" s="53">
+      <c r="E11" s="49">
         <v>355</v>
       </c>
-      <c r="F11" s="53">
+      <c r="F11" s="49">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G11" s="53">
+      <c r="G11" s="49">
         <v>305</v>
       </c>
-      <c r="H11" s="53">
+      <c r="H11" s="49">
         <v>315</v>
       </c>
-      <c r="I11" s="56">
+      <c r="I11" s="52">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="J11" s="54">
+      <c r="J11" s="50">
         <f t="shared" si="2"/>
         <v>0.47</v>
       </c>
-      <c r="K11" s="54">
-        <v>0</v>
-      </c>
-      <c r="L11" s="55">
-        <v>0</v>
-      </c>
-      <c r="M11" s="54">
+      <c r="K11" s="50">
+        <v>0</v>
+      </c>
+      <c r="L11" s="51">
+        <v>0</v>
+      </c>
+      <c r="M11" s="50">
         <f t="shared" si="5"/>
         <v>0.37</v>
       </c>
-      <c r="N11" s="54">
-        <v>0</v>
-      </c>
-      <c r="O11" s="55">
-        <v>0</v>
-      </c>
-      <c r="P11" s="55">
+      <c r="N11" s="50">
+        <v>0</v>
+      </c>
+      <c r="O11" s="51">
+        <v>0</v>
+      </c>
+      <c r="P11" s="51">
         <v>0.72</v>
       </c>
-      <c r="Q11" s="53">
+      <c r="Q11" s="49">
         <v>1</v>
       </c>
-      <c r="R11" s="53">
+      <c r="R11" s="49">
         <v>-130</v>
       </c>
-      <c r="S11" s="53">
+      <c r="S11" s="49">
         <v>-160</v>
       </c>
-      <c r="T11" s="53">
+      <c r="T11" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="53">
+      <c r="A12" s="49">
         <v>100</v>
       </c>
-      <c r="B12" s="53">
+      <c r="B12" s="49">
         <v>60</v>
       </c>
-      <c r="C12" s="53">
-        <v>0</v>
-      </c>
-      <c r="D12" s="53">
+      <c r="C12" s="49">
+        <v>0</v>
+      </c>
+      <c r="D12" s="49">
         <v>353</v>
       </c>
-      <c r="E12" s="53">
+      <c r="E12" s="49">
         <v>358</v>
       </c>
-      <c r="F12" s="53">
+      <c r="F12" s="49">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="G12" s="53">
+      <c r="G12" s="49">
         <v>306</v>
       </c>
-      <c r="H12" s="53">
+      <c r="H12" s="49">
         <v>321</v>
       </c>
-      <c r="I12" s="56">
+      <c r="I12" s="52">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="J12" s="54">
+      <c r="J12" s="50">
         <f t="shared" si="2"/>
         <v>0.47</v>
       </c>
-      <c r="K12" s="54">
+      <c r="K12" s="50">
         <f>(J11-J12)/J11</f>
         <v>0</v>
       </c>
-      <c r="L12" s="55">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="M12" s="54">
+      <c r="L12" s="51">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="M12" s="50">
         <f t="shared" si="5"/>
         <v>0.32</v>
       </c>
-      <c r="N12" s="54">
+      <c r="N12" s="50">
         <f>(M11-M12)/M11</f>
         <v>0.13513513513513511</v>
       </c>
-      <c r="O12" s="55">
+      <c r="O12" s="51">
         <f t="shared" si="4"/>
         <v>13.513513513513512</v>
       </c>
-      <c r="P12" s="55">
+      <c r="P12" s="51">
         <v>0.75</v>
       </c>
-      <c r="Q12" s="53">
+      <c r="Q12" s="49">
         <v>1</v>
       </c>
-      <c r="R12" s="53">
+      <c r="R12" s="49">
         <v>-120</v>
       </c>
-      <c r="S12" s="53">
+      <c r="S12" s="49">
         <v>-130</v>
       </c>
-      <c r="T12" s="53">
+      <c r="T12" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="53">
+      <c r="A13" s="49">
         <v>100</v>
       </c>
-      <c r="B13" s="53">
+      <c r="B13" s="49">
         <v>30</v>
       </c>
-      <c r="C13" s="53">
-        <v>0</v>
-      </c>
-      <c r="D13" s="53">
+      <c r="C13" s="49">
+        <v>0</v>
+      </c>
+      <c r="D13" s="49">
         <v>346</v>
       </c>
-      <c r="E13" s="53">
+      <c r="E13" s="49">
         <v>357</v>
       </c>
-      <c r="F13" s="53">
+      <c r="F13" s="49">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="G13" s="53">
+      <c r="G13" s="49">
         <v>306</v>
       </c>
-      <c r="H13" s="53">
+      <c r="H13" s="49">
         <v>325</v>
       </c>
-      <c r="I13" s="56">
+      <c r="I13" s="52">
         <f t="shared" si="1"/>
         <v>19</v>
       </c>
-      <c r="J13" s="54">
+      <c r="J13" s="50">
         <f t="shared" si="2"/>
         <v>0.4</v>
       </c>
-      <c r="K13" s="54">
+      <c r="K13" s="50">
         <f>(J11-J13)/J11</f>
         <v>0.14893617021276587</v>
       </c>
-      <c r="L13" s="55">
+      <c r="L13" s="51">
         <f t="shared" si="3"/>
         <v>14.893617021276587</v>
       </c>
-      <c r="M13" s="54">
+      <c r="M13" s="50">
         <f t="shared" si="5"/>
         <v>0.79</v>
       </c>
-      <c r="N13" s="54">
+      <c r="N13" s="50">
         <f>(M11-M13)/M11</f>
         <v>-1.1351351351351353</v>
       </c>
-      <c r="O13" s="55">
+      <c r="O13" s="51">
         <f t="shared" si="4"/>
         <v>-113.51351351351353</v>
       </c>
-      <c r="P13" s="55">
+      <c r="P13" s="51">
         <v>0.45</v>
       </c>
-      <c r="Q13" s="53">
+      <c r="Q13" s="49">
         <v>1</v>
       </c>
-      <c r="R13" s="53">
+      <c r="R13" s="49">
         <v>-250</v>
       </c>
-      <c r="S13" s="53">
+      <c r="S13" s="49">
         <v>-280</v>
       </c>
-      <c r="T13" s="53">
+      <c r="T13" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="53">
+      <c r="A14" s="49">
         <v>100</v>
       </c>
-      <c r="B14" s="53">
-        <v>0</v>
-      </c>
-      <c r="C14" s="53">
-        <v>0</v>
-      </c>
-      <c r="D14" s="53">
+      <c r="B14" s="49">
+        <v>0</v>
+      </c>
+      <c r="C14" s="49">
+        <v>0</v>
+      </c>
+      <c r="D14" s="49">
         <v>350</v>
       </c>
-      <c r="E14" s="53">
+      <c r="E14" s="49">
         <v>385</v>
       </c>
-      <c r="F14" s="53">
+      <c r="F14" s="49">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="G14" s="53">
+      <c r="G14" s="49">
         <v>302</v>
       </c>
-      <c r="H14" s="53">
+      <c r="H14" s="49">
         <v>306</v>
       </c>
-      <c r="I14" s="56">
+      <c r="I14" s="52">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="J14" s="54">
+      <c r="J14" s="50">
         <f t="shared" si="2"/>
         <v>0.48</v>
       </c>
-      <c r="K14" s="54">
+      <c r="K14" s="50">
         <f>(J11-J14)/J11</f>
         <v>-2.1276595744680871E-2</v>
       </c>
-      <c r="L14" s="55">
+      <c r="L14" s="51">
         <f t="shared" si="3"/>
         <v>-2.1276595744680873</v>
       </c>
-      <c r="M14" s="54">
+      <c r="M14" s="50">
         <f t="shared" si="5"/>
         <v>0.34166666666666667</v>
       </c>
-      <c r="N14" s="54">
+      <c r="N14" s="50">
         <f>(M11-M14)/M11</f>
         <v>7.6576576576576544E-2</v>
       </c>
-      <c r="O14" s="55">
+      <c r="O14" s="51">
         <f t="shared" si="4"/>
         <v>7.657657657657654</v>
       </c>
-      <c r="P14" s="55">
+      <c r="P14" s="51">
         <v>0.67</v>
       </c>
-      <c r="Q14" s="55">
+      <c r="Q14" s="51">
         <v>0.69</v>
       </c>
-      <c r="R14" s="53">
+      <c r="R14" s="49">
         <v>-270</v>
       </c>
-      <c r="S14" s="53">
+      <c r="S14" s="49">
         <v>-370</v>
       </c>
-      <c r="T14" s="53">
+      <c r="T14" s="49">
         <v>-240</v>
       </c>
     </row>
     <row r="15" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="53">
+      <c r="A15" s="49">
         <v>120</v>
       </c>
-      <c r="B15" s="53">
+      <c r="B15" s="49">
         <v>90</v>
       </c>
-      <c r="C15" s="53">
-        <v>0</v>
-      </c>
-      <c r="D15" s="53">
+      <c r="C15" s="49">
+        <v>0</v>
+      </c>
+      <c r="D15" s="49">
         <v>353</v>
       </c>
-      <c r="E15" s="53">
+      <c r="E15" s="49">
         <v>356</v>
       </c>
-      <c r="F15" s="53">
+      <c r="F15" s="49">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G15" s="53">
+      <c r="G15" s="49">
         <v>304</v>
       </c>
-      <c r="H15" s="53">
+      <c r="H15" s="49">
         <v>315</v>
       </c>
-      <c r="I15" s="56">
+      <c r="I15" s="52">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="J15" s="54">
+      <c r="J15" s="50">
         <f t="shared" si="2"/>
         <v>0.40833333333333333</v>
       </c>
-      <c r="K15" s="54">
-        <v>0</v>
-      </c>
-      <c r="L15" s="55">
-        <v>0</v>
-      </c>
-      <c r="M15" s="54">
+      <c r="K15" s="50">
+        <v>0</v>
+      </c>
+      <c r="L15" s="51">
+        <v>0</v>
+      </c>
+      <c r="M15" s="50">
         <f t="shared" si="5"/>
         <v>0.35833333333333334</v>
       </c>
-      <c r="N15" s="54">
-        <v>0</v>
-      </c>
-      <c r="O15" s="55">
-        <v>0</v>
-      </c>
-      <c r="P15" s="55">
+      <c r="N15" s="50">
+        <v>0</v>
+      </c>
+      <c r="O15" s="51">
+        <v>0</v>
+      </c>
+      <c r="P15" s="51">
         <v>0.77</v>
       </c>
-      <c r="Q15" s="53">
+      <c r="Q15" s="49">
         <v>1</v>
       </c>
-      <c r="R15" s="53">
+      <c r="R15" s="49">
         <v>-100</v>
       </c>
-      <c r="S15" s="53">
+      <c r="S15" s="49">
         <v>-130</v>
       </c>
-      <c r="T15" s="53">
+      <c r="T15" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="53">
+      <c r="A16" s="49">
         <v>120</v>
       </c>
-      <c r="B16" s="53">
+      <c r="B16" s="49">
         <v>60</v>
       </c>
-      <c r="C16" s="53">
-        <v>0</v>
-      </c>
-      <c r="D16" s="53">
+      <c r="C16" s="49">
+        <v>0</v>
+      </c>
+      <c r="D16" s="49">
         <v>353</v>
       </c>
-      <c r="E16" s="53">
+      <c r="E16" s="49">
         <v>356</v>
       </c>
-      <c r="F16" s="53">
+      <c r="F16" s="49">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G16" s="53">
+      <c r="G16" s="49">
         <v>307</v>
       </c>
-      <c r="H16" s="53">
+      <c r="H16" s="49">
         <v>313</v>
       </c>
-      <c r="I16" s="56">
+      <c r="I16" s="52">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="J16" s="54">
+      <c r="J16" s="50">
         <f t="shared" si="2"/>
         <v>0.38333333333333336</v>
       </c>
-      <c r="K16" s="54">
+      <c r="K16" s="50">
         <f>(J15-J16)/J15</f>
         <v>6.122448979591829E-2</v>
       </c>
-      <c r="L16" s="55">
+      <c r="L16" s="51">
         <f t="shared" si="3"/>
         <v>6.1224489795918293</v>
       </c>
-      <c r="M16" s="54">
+      <c r="M16" s="50">
         <f t="shared" si="5"/>
         <v>0.29166666666666669</v>
       </c>
-      <c r="N16" s="54">
+      <c r="N16" s="50">
         <f>(M15-M16)/M15</f>
         <v>0.18604651162790695</v>
       </c>
-      <c r="O16" s="55">
+      <c r="O16" s="51">
         <f t="shared" si="4"/>
         <v>18.604651162790695</v>
       </c>
-      <c r="P16" s="55">
+      <c r="P16" s="51">
         <v>0.8</v>
       </c>
-      <c r="Q16" s="53">
+      <c r="Q16" s="49">
         <v>1</v>
       </c>
-      <c r="R16" s="53">
+      <c r="R16" s="49">
         <v>-75</v>
       </c>
-      <c r="S16" s="53">
+      <c r="S16" s="49">
         <v>-85</v>
       </c>
-      <c r="T16" s="53">
+      <c r="T16" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="53">
+      <c r="A17" s="49">
         <v>120</v>
       </c>
-      <c r="B17" s="53">
+      <c r="B17" s="49">
         <v>30</v>
       </c>
-      <c r="C17" s="53">
-        <v>0</v>
-      </c>
-      <c r="D17" s="53">
+      <c r="C17" s="49">
+        <v>0</v>
+      </c>
+      <c r="D17" s="49">
         <v>348</v>
       </c>
-      <c r="E17" s="53">
+      <c r="E17" s="49">
         <v>358</v>
       </c>
-      <c r="F17" s="53">
+      <c r="F17" s="49">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="G17" s="53">
+      <c r="G17" s="49">
         <v>303</v>
       </c>
-      <c r="H17" s="53">
+      <c r="H17" s="49">
         <v>323</v>
       </c>
-      <c r="I17" s="56">
+      <c r="I17" s="52">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="J17" s="54">
+      <c r="J17" s="50">
         <f t="shared" si="2"/>
         <v>0.375</v>
       </c>
-      <c r="K17" s="54">
+      <c r="K17" s="50">
         <f>(J15-J17)/J15</f>
         <v>8.1632653061224469E-2</v>
       </c>
-      <c r="L17" s="55">
+      <c r="L17" s="51">
         <f t="shared" si="3"/>
         <v>8.1632653061224474</v>
       </c>
-      <c r="M17" s="54">
+      <c r="M17" s="50">
         <f t="shared" si="5"/>
         <v>1.2375</v>
       </c>
-      <c r="N17" s="54">
+      <c r="N17" s="50">
         <f>(M15-M17)/M15</f>
         <v>-2.4534883720930232</v>
       </c>
-      <c r="O17" s="55">
+      <c r="O17" s="51">
         <f t="shared" si="4"/>
         <v>-245.3488372093023</v>
       </c>
-      <c r="P17" s="55">
+      <c r="P17" s="51">
         <v>0.6</v>
       </c>
-      <c r="Q17" s="53">
+      <c r="Q17" s="49">
         <v>1</v>
       </c>
-      <c r="R17" s="53">
+      <c r="R17" s="49">
         <v>-185</v>
       </c>
-      <c r="S17" s="53">
+      <c r="S17" s="49">
         <v>-230</v>
       </c>
-      <c r="T17" s="53">
+      <c r="T17" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="53">
+      <c r="A18" s="49">
         <v>40</v>
       </c>
-      <c r="B18" s="53">
+      <c r="B18" s="49">
         <v>90</v>
       </c>
-      <c r="C18" s="53">
+      <c r="C18" s="49">
         <v>90</v>
       </c>
-      <c r="D18" s="53">
+      <c r="D18" s="49">
         <v>342</v>
       </c>
-      <c r="E18" s="53">
+      <c r="E18" s="49">
         <v>355</v>
       </c>
-      <c r="F18" s="53">
+      <c r="F18" s="49">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="G18" s="55">
+      <c r="G18" s="51">
         <v>304.5</v>
       </c>
-      <c r="H18" s="55">
+      <c r="H18" s="51">
         <v>305.5</v>
       </c>
-      <c r="I18" s="56">
+      <c r="I18" s="52">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J18" s="54">
+      <c r="J18" s="50">
         <f t="shared" si="2"/>
         <v>0.9375</v>
       </c>
-      <c r="K18" s="54">
+      <c r="K18" s="50">
         <f>(J2-J18)/J2</f>
         <v>0.10714285714285718</v>
       </c>
-      <c r="L18" s="55">
+      <c r="L18" s="51">
         <f t="shared" si="3"/>
         <v>10.714285714285717</v>
       </c>
-      <c r="M18" s="54">
+      <c r="M18" s="50">
         <f t="shared" ref="M18:M31" si="6">(E18-H18)/A18</f>
         <v>1.2375</v>
       </c>
-      <c r="N18" s="54">
+      <c r="N18" s="50">
         <f>(M2-M18)/M2</f>
         <v>-0.33783783783783783</v>
       </c>
-      <c r="O18" s="55">
+      <c r="O18" s="51">
         <f t="shared" si="4"/>
         <v>-33.783783783783782</v>
       </c>
-      <c r="P18" s="55">
+      <c r="P18" s="51">
         <v>0.5</v>
       </c>
-      <c r="Q18" s="55">
+      <c r="Q18" s="51">
         <v>0.57999999999999996</v>
       </c>
-      <c r="R18" s="53">
+      <c r="R18" s="49">
         <v>-220</v>
       </c>
-      <c r="S18" s="53">
+      <c r="S18" s="49">
         <v>-235</v>
       </c>
-      <c r="T18" s="53">
+      <c r="T18" s="49">
         <v>-225</v>
       </c>
     </row>
     <row r="19" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="53">
+      <c r="A19" s="49">
         <v>40</v>
       </c>
-      <c r="B19" s="53">
+      <c r="B19" s="49">
         <v>90</v>
       </c>
-      <c r="C19" s="53">
+      <c r="C19" s="49">
         <v>60</v>
       </c>
-      <c r="D19" s="53">
+      <c r="D19" s="49">
         <v>347</v>
       </c>
-      <c r="E19" s="53">
+      <c r="E19" s="49">
         <v>352</v>
       </c>
-      <c r="F19" s="53">
+      <c r="F19" s="49">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="G19" s="53">
+      <c r="G19" s="49">
         <v>305</v>
       </c>
-      <c r="H19" s="53">
+      <c r="H19" s="49">
         <v>307</v>
       </c>
-      <c r="I19" s="56">
+      <c r="I19" s="52">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="J19" s="54">
+      <c r="J19" s="50">
         <f t="shared" si="2"/>
         <v>1.05</v>
       </c>
-      <c r="K19" s="54">
+      <c r="K19" s="50">
         <f>(J2-J19)/J2</f>
         <v>0</v>
       </c>
-      <c r="L19" s="55">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="M19" s="54">
+      <c r="L19" s="51">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="M19" s="50">
         <f t="shared" si="6"/>
         <v>1.125</v>
       </c>
-      <c r="N19" s="54">
+      <c r="N19" s="50">
         <f>(M2-M19)/M2</f>
         <v>-0.21621621621621614</v>
       </c>
-      <c r="O19" s="55">
+      <c r="O19" s="51">
         <f t="shared" si="4"/>
         <v>-21.621621621621614</v>
       </c>
-      <c r="P19" s="55">
+      <c r="P19" s="51">
         <v>0.6</v>
       </c>
-      <c r="Q19" s="55">
+      <c r="Q19" s="51">
         <v>0.72</v>
       </c>
-      <c r="R19" s="53">
+      <c r="R19" s="49">
         <v>-175</v>
       </c>
-      <c r="S19" s="53">
+      <c r="S19" s="49">
         <v>-190</v>
       </c>
-      <c r="T19" s="53">
+      <c r="T19" s="49">
         <v>-120</v>
       </c>
     </row>
     <row r="20" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="53">
+      <c r="A20" s="49">
         <v>40</v>
       </c>
-      <c r="B20" s="53">
+      <c r="B20" s="49">
         <v>90</v>
       </c>
-      <c r="C20" s="53">
+      <c r="C20" s="49">
         <v>30</v>
       </c>
-      <c r="D20" s="53">
+      <c r="D20" s="49">
         <v>350</v>
       </c>
-      <c r="E20" s="53">
+      <c r="E20" s="49">
         <v>354</v>
       </c>
-      <c r="F20" s="53">
+      <c r="F20" s="49">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G20" s="53">
+      <c r="G20" s="49">
         <v>305</v>
       </c>
-      <c r="H20" s="53">
+      <c r="H20" s="49">
         <v>306</v>
       </c>
-      <c r="I20" s="56">
+      <c r="I20" s="52">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="J20" s="54">
+      <c r="J20" s="50">
         <f t="shared" si="2"/>
         <v>1.125</v>
       </c>
-      <c r="K20" s="54">
+      <c r="K20" s="50">
         <f>(J2-J20)/J2</f>
         <v>-7.1428571428571383E-2</v>
       </c>
-      <c r="L20" s="55">
+      <c r="L20" s="51">
         <f t="shared" si="3"/>
         <v>-7.1428571428571379</v>
       </c>
-      <c r="M20" s="54">
+      <c r="M20" s="50">
         <f t="shared" si="6"/>
         <v>1.2</v>
       </c>
-      <c r="N20" s="54">
+      <c r="N20" s="50">
         <f>(M2-M20)/M2</f>
         <v>-0.2972972972972972</v>
       </c>
-      <c r="O20" s="55">
+      <c r="O20" s="51">
         <f t="shared" si="4"/>
         <v>-29.729729729729719</v>
       </c>
-      <c r="P20" s="55">
+      <c r="P20" s="51">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q20" s="55">
+      <c r="Q20" s="51">
         <v>0.6</v>
       </c>
-      <c r="R20" s="53">
+      <c r="R20" s="49">
         <v>-230</v>
       </c>
-      <c r="S20" s="53">
+      <c r="S20" s="49">
         <v>-240</v>
       </c>
-      <c r="T20" s="53">
+      <c r="T20" s="49">
         <v>-220</v>
       </c>
     </row>
     <row r="21" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="53">
+      <c r="A21" s="49">
         <v>60</v>
       </c>
-      <c r="B21" s="53">
+      <c r="B21" s="49">
         <v>90</v>
       </c>
-      <c r="C21" s="53">
+      <c r="C21" s="49">
         <v>90</v>
       </c>
-      <c r="D21" s="53">
+      <c r="D21" s="49">
         <v>345</v>
       </c>
-      <c r="E21" s="53">
+      <c r="E21" s="49">
         <v>368</v>
       </c>
-      <c r="F21" s="53">
+      <c r="F21" s="49">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="G21" s="55">
+      <c r="G21" s="51">
         <v>304.5</v>
       </c>
-      <c r="H21" s="55">
+      <c r="H21" s="51">
         <v>307.5</v>
       </c>
-      <c r="I21" s="56">
+      <c r="I21" s="52">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="J21" s="54">
+      <c r="J21" s="50">
         <f t="shared" si="2"/>
         <v>0.67500000000000004</v>
       </c>
-      <c r="K21" s="54"/>
-      <c r="L21" s="55"/>
-      <c r="M21" s="54">
+      <c r="K21" s="50"/>
+      <c r="L21" s="51"/>
+      <c r="M21" s="50">
         <f t="shared" si="6"/>
         <v>1.0083333333333333</v>
       </c>
-      <c r="N21" s="54"/>
-      <c r="O21" s="55"/>
-      <c r="P21" s="55">
+      <c r="N21" s="50"/>
+      <c r="O21" s="51"/>
+      <c r="P21" s="51">
         <v>0.62</v>
       </c>
-      <c r="Q21" s="55">
+      <c r="Q21" s="51">
         <v>0.8</v>
       </c>
-      <c r="R21" s="53">
+      <c r="R21" s="49">
         <v>-155</v>
       </c>
-      <c r="S21" s="53">
+      <c r="S21" s="49">
         <v>-175</v>
       </c>
-      <c r="T21" s="53">
+      <c r="T21" s="49">
         <v>-90</v>
       </c>
     </row>
     <row r="22" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="53">
+      <c r="A22" s="49">
         <v>60</v>
       </c>
-      <c r="B22" s="53">
+      <c r="B22" s="49">
         <v>90</v>
       </c>
-      <c r="C22" s="53">
+      <c r="C22" s="49">
         <v>60</v>
       </c>
-      <c r="D22" s="53">
+      <c r="D22" s="49">
         <v>342</v>
       </c>
-      <c r="E22" s="53">
+      <c r="E22" s="49">
         <v>351</v>
       </c>
-      <c r="F22" s="53">
+      <c r="F22" s="49">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="G22" s="53">
+      <c r="G22" s="49">
         <v>305</v>
       </c>
-      <c r="H22" s="53">
+      <c r="H22" s="49">
         <v>320</v>
       </c>
-      <c r="I22" s="56">
+      <c r="I22" s="52">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="J22" s="54">
+      <c r="J22" s="50">
         <f t="shared" si="2"/>
         <v>0.6166666666666667</v>
       </c>
-      <c r="K22" s="54"/>
-      <c r="L22" s="55"/>
-      <c r="M22" s="54">
+      <c r="K22" s="50"/>
+      <c r="L22" s="51"/>
+      <c r="M22" s="50">
         <f t="shared" si="6"/>
         <v>0.51666666666666672</v>
       </c>
-      <c r="N22" s="54"/>
-      <c r="O22" s="55"/>
-      <c r="P22" s="55">
+      <c r="N22" s="50"/>
+      <c r="O22" s="51"/>
+      <c r="P22" s="51">
         <v>0.5</v>
       </c>
-      <c r="Q22" s="55">
+      <c r="Q22" s="51">
         <v>0.74</v>
       </c>
-      <c r="R22" s="53">
+      <c r="R22" s="49">
         <v>-220</v>
       </c>
-      <c r="S22" s="53">
+      <c r="S22" s="49">
         <v>-225</v>
       </c>
-      <c r="T22" s="53">
+      <c r="T22" s="49">
         <v>-75</v>
       </c>
     </row>
     <row r="23" spans="1:20" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="53">
+      <c r="A23" s="49">
         <v>60</v>
       </c>
-      <c r="B23" s="53">
+      <c r="B23" s="49">
         <v>90</v>
       </c>
-      <c r="C23" s="53">
+      <c r="C23" s="49">
         <v>30</v>
       </c>
-      <c r="D23" s="53">
+      <c r="D23" s="49">
         <v>351</v>
       </c>
-      <c r="E23" s="53">
+      <c r="E23" s="49">
         <v>354</v>
       </c>
-      <c r="F23" s="53">
+      <c r="F23" s="49">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G23" s="53">
+      <c r="G23" s="49">
         <v>307</v>
       </c>
-      <c r="H23" s="53">
+      <c r="H23" s="49">
         <v>319</v>
       </c>
-      <c r="I23" s="56">
+      <c r="I23" s="52">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="J23" s="54">
+      <c r="J23" s="50">
         <f t="shared" si="2"/>
         <v>0.73333333333333328</v>
       </c>
-      <c r="K23" s="54"/>
-      <c r="L23" s="55"/>
-      <c r="M23" s="54">
+      <c r="K23" s="50"/>
+      <c r="L23" s="51"/>
+      <c r="M23" s="50">
         <f t="shared" si="6"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="N23" s="54"/>
-      <c r="O23" s="55"/>
-      <c r="P23" s="55">
+      <c r="N23" s="50"/>
+      <c r="O23" s="51"/>
+      <c r="P23" s="51">
         <v>0.68</v>
       </c>
-      <c r="Q23" s="55">
+      <c r="Q23" s="51">
         <v>0.78</v>
       </c>
-      <c r="R23" s="53">
+      <c r="R23" s="49">
         <v>-130</v>
       </c>
-      <c r="S23" s="53">
+      <c r="S23" s="49">
         <v>-260</v>
       </c>
-      <c r="T23" s="53">
+      <c r="T23" s="49">
         <v>-70</v>
       </c>
     </row>
     <row r="24" spans="1:20" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="53">
+      <c r="A24" s="49">
         <v>80</v>
       </c>
-      <c r="B24" s="53">
+      <c r="B24" s="49">
         <v>90</v>
       </c>
-      <c r="C24" s="53">
+      <c r="C24" s="49">
         <v>60</v>
       </c>
-      <c r="D24" s="53">
+      <c r="D24" s="49">
         <v>348</v>
       </c>
-      <c r="E24" s="53">
+      <c r="E24" s="49">
         <v>360</v>
       </c>
-      <c r="F24" s="53">
+      <c r="F24" s="49">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="G24" s="53">
+      <c r="G24" s="49">
         <v>304</v>
       </c>
-      <c r="H24" s="53">
+      <c r="H24" s="49">
         <v>329</v>
       </c>
-      <c r="I24" s="56">
+      <c r="I24" s="52">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="J24" s="54">
+      <c r="J24" s="50">
         <f t="shared" si="2"/>
         <v>0.55000000000000004</v>
       </c>
-      <c r="K24" s="54">
+      <c r="K24" s="50">
         <f>(J7-J24)/J7</f>
         <v>8.3333333333333232E-2</v>
       </c>
-      <c r="L24" s="55">
+      <c r="L24" s="51">
         <f t="shared" si="3"/>
         <v>8.3333333333333233</v>
       </c>
-      <c r="M24" s="54">
+      <c r="M24" s="50">
         <f t="shared" si="6"/>
         <v>0.38750000000000001</v>
       </c>
-      <c r="N24" s="54">
+      <c r="N24" s="50">
         <f>(M7-M24)/M7</f>
         <v>0.31111111111111112</v>
       </c>
-      <c r="O24" s="55">
+      <c r="O24" s="51">
         <f t="shared" si="4"/>
         <v>31.111111111111111</v>
       </c>
-      <c r="P24" s="55">
+      <c r="P24" s="51">
         <v>0.62</v>
       </c>
-      <c r="Q24" s="53">
+      <c r="Q24" s="49">
         <v>1</v>
       </c>
-      <c r="R24" s="53">
+      <c r="R24" s="49">
         <v>-160</v>
       </c>
-      <c r="S24" s="53">
+      <c r="S24" s="49">
         <v>-230</v>
       </c>
-      <c r="T24" s="53">
+      <c r="T24" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:20" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="53">
+      <c r="A25" s="49">
         <v>80</v>
       </c>
-      <c r="B25" s="53">
+      <c r="B25" s="49">
         <v>90</v>
       </c>
-      <c r="C25" s="53">
+      <c r="C25" s="49">
         <v>30</v>
       </c>
-      <c r="D25" s="53">
+      <c r="D25" s="49">
         <v>346</v>
       </c>
-      <c r="E25" s="53">
+      <c r="E25" s="49">
         <v>354</v>
       </c>
-      <c r="F25" s="53">
+      <c r="F25" s="49">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="G25" s="53">
+      <c r="G25" s="49">
         <v>304</v>
       </c>
-      <c r="H25" s="53">
+      <c r="H25" s="49">
         <v>326</v>
       </c>
-      <c r="I25" s="56">
+      <c r="I25" s="52">
         <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="J25" s="54">
+      <c r="J25" s="50">
         <f t="shared" si="2"/>
         <v>0.52500000000000002</v>
       </c>
-      <c r="K25" s="54">
+      <c r="K25" s="50">
         <f>(J7-J25)/J7</f>
         <v>0.12499999999999993</v>
       </c>
-      <c r="L25" s="55">
+      <c r="L25" s="51">
         <f t="shared" si="3"/>
         <v>12.499999999999993</v>
       </c>
-      <c r="M25" s="54">
+      <c r="M25" s="50">
         <f t="shared" si="6"/>
         <v>0.35</v>
       </c>
-      <c r="N25" s="54">
+      <c r="N25" s="50">
         <f>(M7-M25)/M7</f>
         <v>0.37777777777777782</v>
       </c>
-      <c r="O25" s="55">
+      <c r="O25" s="51">
         <f t="shared" si="4"/>
         <v>37.777777777777786</v>
       </c>
-      <c r="P25" s="55">
+      <c r="P25" s="51">
         <v>0.46</v>
       </c>
-      <c r="Q25" s="55">
+      <c r="Q25" s="51">
         <v>0.92</v>
       </c>
-      <c r="R25" s="53">
+      <c r="R25" s="49">
         <v>-255</v>
       </c>
-      <c r="S25" s="53">
+      <c r="S25" s="49">
         <v>-300</v>
       </c>
-      <c r="T25" s="53">
+      <c r="T25" s="49">
         <v>-20</v>
       </c>
     </row>
     <row r="26" spans="1:20" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="53">
+      <c r="A26" s="49">
         <v>100</v>
       </c>
-      <c r="B26" s="53">
+      <c r="B26" s="49">
         <v>90</v>
       </c>
-      <c r="C26" s="53">
+      <c r="C26" s="49">
         <v>90</v>
       </c>
-      <c r="D26" s="53">
+      <c r="D26" s="49">
         <v>352</v>
       </c>
-      <c r="E26" s="53">
+      <c r="E26" s="49">
         <v>374</v>
       </c>
-      <c r="F26" s="53">
+      <c r="F26" s="49">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="G26" s="53">
+      <c r="G26" s="49">
         <v>306</v>
       </c>
-      <c r="H26" s="53">
+      <c r="H26" s="49">
         <v>308</v>
       </c>
-      <c r="I26" s="56">
+      <c r="I26" s="52">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="J26" s="54">
+      <c r="J26" s="50">
         <f t="shared" si="2"/>
         <v>0.46</v>
       </c>
-      <c r="K26" s="54">
+      <c r="K26" s="50">
         <f>(J11-J26)/J11</f>
         <v>2.1276595744680753E-2</v>
       </c>
-      <c r="L26" s="55">
+      <c r="L26" s="51">
         <f t="shared" si="3"/>
         <v>2.1276595744680753</v>
       </c>
-      <c r="M26" s="54">
+      <c r="M26" s="50">
         <f t="shared" si="6"/>
         <v>0.66</v>
       </c>
-      <c r="N26" s="54">
+      <c r="N26" s="50">
         <f>(M11-M26)/M11</f>
         <v>-0.78378378378378388</v>
       </c>
-      <c r="O26" s="55">
+      <c r="O26" s="51">
         <f t="shared" si="4"/>
         <v>-78.378378378378386</v>
       </c>
-      <c r="P26" s="55">
+      <c r="P26" s="51">
         <v>0.55000000000000004</v>
       </c>
-      <c r="Q26" s="53">
+      <c r="Q26" s="49">
         <v>1</v>
       </c>
-      <c r="R26" s="53">
+      <c r="R26" s="49">
         <v>-150</v>
       </c>
-      <c r="S26" s="53">
+      <c r="S26" s="49">
         <v>-170</v>
       </c>
-      <c r="T26" s="53">
+      <c r="T26" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:20" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="53">
+      <c r="A27" s="49">
         <v>100</v>
       </c>
-      <c r="B27" s="53">
+      <c r="B27" s="49">
         <v>90</v>
       </c>
-      <c r="C27" s="53">
+      <c r="C27" s="49">
         <v>60</v>
       </c>
-      <c r="D27" s="53">
+      <c r="D27" s="49">
         <v>341</v>
       </c>
-      <c r="E27" s="53">
+      <c r="E27" s="49">
         <v>357</v>
       </c>
-      <c r="F27" s="53">
+      <c r="F27" s="49">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="G27" s="53">
+      <c r="G27" s="49">
         <v>302</v>
       </c>
-      <c r="H27" s="53">
+      <c r="H27" s="49">
         <v>330</v>
       </c>
-      <c r="I27" s="56">
+      <c r="I27" s="52">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="J27" s="54">
+      <c r="J27" s="50">
         <f t="shared" si="2"/>
         <v>0.39</v>
       </c>
-      <c r="K27" s="54">
+      <c r="K27" s="50">
         <f>(J11-J27)/J11</f>
         <v>0.17021276595744672</v>
       </c>
-      <c r="L27" s="55">
+      <c r="L27" s="51">
         <f t="shared" si="3"/>
         <v>17.021276595744673</v>
       </c>
-      <c r="M27" s="54">
+      <c r="M27" s="50">
         <f t="shared" si="6"/>
         <v>0.27</v>
       </c>
-      <c r="N27" s="54">
+      <c r="N27" s="50">
         <f>(M11-M27)/M11</f>
         <v>0.27027027027027023</v>
       </c>
-      <c r="O27" s="55">
+      <c r="O27" s="51">
         <f t="shared" si="4"/>
         <v>27.027027027027025</v>
       </c>
-      <c r="P27" s="55">
+      <c r="P27" s="51">
         <v>0.48</v>
       </c>
-      <c r="Q27" s="53">
+      <c r="Q27" s="49">
         <v>1</v>
       </c>
-      <c r="R27" s="53">
+      <c r="R27" s="49">
         <v>-220</v>
       </c>
-      <c r="S27" s="53">
+      <c r="S27" s="49">
         <v>-250</v>
       </c>
-      <c r="T27" s="53">
+      <c r="T27" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:20" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="53">
+      <c r="A28" s="49">
         <v>100</v>
       </c>
-      <c r="B28" s="53">
+      <c r="B28" s="49">
         <v>90</v>
       </c>
-      <c r="C28" s="53">
+      <c r="C28" s="49">
         <v>30</v>
       </c>
-      <c r="D28" s="53">
+      <c r="D28" s="49">
         <v>346</v>
       </c>
-      <c r="E28" s="53">
+      <c r="E28" s="49">
         <v>355</v>
       </c>
-      <c r="F28" s="53">
+      <c r="F28" s="49">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="G28" s="53">
+      <c r="G28" s="49">
         <v>306</v>
       </c>
-      <c r="H28" s="53">
+      <c r="H28" s="49">
         <v>329</v>
       </c>
-      <c r="I28" s="56">
+      <c r="I28" s="52">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="J28" s="54">
+      <c r="J28" s="50">
         <f t="shared" si="2"/>
         <v>0.4</v>
       </c>
-      <c r="K28" s="54">
+      <c r="K28" s="50">
         <f>(J11-J28)/J11</f>
         <v>0.14893617021276587</v>
       </c>
-      <c r="L28" s="55">
+      <c r="L28" s="51">
         <f t="shared" si="3"/>
         <v>14.893617021276587</v>
       </c>
-      <c r="M28" s="54">
+      <c r="M28" s="50">
         <f t="shared" si="6"/>
         <v>0.26</v>
       </c>
-      <c r="N28" s="54">
+      <c r="N28" s="50">
         <f>(M11-M28)/M11</f>
         <v>0.29729729729729726</v>
       </c>
-      <c r="O28" s="55">
+      <c r="O28" s="51">
         <f t="shared" si="4"/>
         <v>29.729729729729726</v>
       </c>
-      <c r="P28" s="55">
+      <c r="P28" s="51">
         <v>0.6</v>
       </c>
-      <c r="Q28" s="53">
+      <c r="Q28" s="49">
         <v>1</v>
       </c>
-      <c r="R28" s="53">
+      <c r="R28" s="49">
         <v>-150</v>
       </c>
-      <c r="S28" s="53">
+      <c r="S28" s="49">
         <v>-210</v>
       </c>
-      <c r="T28" s="53">
+      <c r="T28" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:20" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="53">
+      <c r="A29" s="49">
         <v>120</v>
       </c>
-      <c r="B29" s="53">
+      <c r="B29" s="49">
         <v>90</v>
       </c>
-      <c r="C29" s="53">
+      <c r="C29" s="49">
         <v>90</v>
       </c>
-      <c r="D29" s="53">
+      <c r="D29" s="49">
         <v>354</v>
       </c>
-      <c r="E29" s="53">
+      <c r="E29" s="49">
         <v>370</v>
       </c>
-      <c r="F29" s="53">
+      <c r="F29" s="49">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="G29" s="53">
+      <c r="G29" s="49">
         <v>304</v>
       </c>
-      <c r="H29" s="53">
+      <c r="H29" s="49">
         <v>314</v>
       </c>
-      <c r="I29" s="56">
+      <c r="I29" s="52">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="J29" s="54">
+      <c r="J29" s="50">
         <f t="shared" si="2"/>
         <v>0.41666666666666669</v>
       </c>
-      <c r="K29" s="54">
+      <c r="K29" s="50">
         <f>(J15-J29)/J15</f>
         <v>-2.0408163265306187E-2</v>
       </c>
-      <c r="L29" s="55">
+      <c r="L29" s="51">
         <f t="shared" si="3"/>
         <v>-2.0408163265306185</v>
       </c>
-      <c r="M29" s="54">
+      <c r="M29" s="50">
         <f t="shared" si="6"/>
         <v>0.46666666666666667</v>
       </c>
-      <c r="N29" s="54">
+      <c r="N29" s="50">
         <f>(M15-M29)/M15</f>
         <v>-0.30232558139534882</v>
       </c>
-      <c r="O29" s="55">
+      <c r="O29" s="51">
         <f t="shared" si="4"/>
         <v>-30.232558139534881</v>
       </c>
-      <c r="P29" s="55">
+      <c r="P29" s="51">
         <v>0.6</v>
       </c>
-      <c r="Q29" s="53">
+      <c r="Q29" s="49">
         <v>1</v>
       </c>
-      <c r="R29" s="53">
+      <c r="R29" s="49">
         <v>215</v>
       </c>
-      <c r="S29" s="53">
+      <c r="S29" s="49">
         <v>-230</v>
       </c>
-      <c r="T29" s="53">
+      <c r="T29" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:20" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="53">
+      <c r="A30" s="49">
         <v>120</v>
       </c>
-      <c r="B30" s="53">
+      <c r="B30" s="49">
         <v>90</v>
       </c>
-      <c r="C30" s="53">
+      <c r="C30" s="49">
         <v>60</v>
       </c>
-      <c r="D30" s="53">
+      <c r="D30" s="49">
         <v>342</v>
       </c>
-      <c r="E30" s="53">
+      <c r="E30" s="49">
         <v>355</v>
       </c>
-      <c r="F30" s="53">
+      <c r="F30" s="49">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="G30" s="53">
+      <c r="G30" s="49">
         <v>302</v>
       </c>
-      <c r="H30" s="53">
+      <c r="H30" s="49">
         <v>330</v>
       </c>
-      <c r="I30" s="56">
+      <c r="I30" s="52">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="J30" s="54">
+      <c r="J30" s="50">
         <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="K30" s="54">
+      <c r="K30" s="50">
         <f>(J15-J30)/J15</f>
         <v>0.18367346938775514</v>
       </c>
-      <c r="L30" s="55">
+      <c r="L30" s="51">
         <f t="shared" si="3"/>
         <v>18.367346938775515</v>
       </c>
-      <c r="M30" s="54">
+      <c r="M30" s="50">
         <f t="shared" si="6"/>
         <v>0.20833333333333334</v>
       </c>
-      <c r="N30" s="54">
+      <c r="N30" s="50">
         <f>(M15-M30)/M15</f>
         <v>0.41860465116279066</v>
       </c>
-      <c r="O30" s="55">
+      <c r="O30" s="51">
         <f t="shared" si="4"/>
         <v>41.860465116279066</v>
       </c>
-      <c r="P30" s="55">
+      <c r="P30" s="51">
         <v>0.54</v>
       </c>
-      <c r="Q30" s="53">
+      <c r="Q30" s="49">
         <v>1</v>
       </c>
-      <c r="R30" s="53">
+      <c r="R30" s="49">
         <v>-215</v>
       </c>
-      <c r="S30" s="53">
+      <c r="S30" s="49">
         <v>-230</v>
       </c>
-      <c r="T30" s="53">
+      <c r="T30" s="49">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:20" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="53">
+      <c r="A31" s="49">
         <v>120</v>
       </c>
-      <c r="B31" s="53">
+      <c r="B31" s="49">
         <v>90</v>
       </c>
-      <c r="C31" s="53">
+      <c r="C31" s="49">
         <v>30</v>
       </c>
-      <c r="D31" s="53">
+      <c r="D31" s="49">
         <v>343</v>
       </c>
-      <c r="E31" s="53">
+      <c r="E31" s="49">
         <v>355</v>
       </c>
-      <c r="F31" s="53">
+      <c r="F31" s="49">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="G31" s="53">
+      <c r="G31" s="49">
         <v>304</v>
       </c>
-      <c r="H31" s="53">
+      <c r="H31" s="49">
         <v>327</v>
       </c>
-      <c r="I31" s="56">
+      <c r="I31" s="52">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="J31" s="54">
+      <c r="J31" s="50">
         <f t="shared" si="2"/>
         <v>0.32500000000000001</v>
       </c>
-      <c r="K31" s="54">
+      <c r="K31" s="50">
         <f>(J15-J31)/J15</f>
         <v>0.20408163265306117</v>
       </c>
-      <c r="L31" s="55">
+      <c r="L31" s="51">
         <f t="shared" si="3"/>
         <v>20.408163265306118</v>
       </c>
-      <c r="M31" s="54">
+      <c r="M31" s="50">
         <f t="shared" si="6"/>
         <v>0.23333333333333334</v>
       </c>
-      <c r="N31" s="54">
+      <c r="N31" s="50">
         <f>(M15-M31)/M15</f>
         <v>0.34883720930232559</v>
       </c>
-      <c r="O31" s="55">
+      <c r="O31" s="51">
         <f t="shared" si="4"/>
         <v>34.883720930232556</v>
       </c>
-      <c r="P31" s="55">
+      <c r="P31" s="51">
         <v>0.52</v>
       </c>
-      <c r="Q31" s="53">
+      <c r="Q31" s="49">
         <v>1</v>
       </c>
-      <c r="R31" s="53">
+      <c r="R31" s="49">
         <v>-200</v>
       </c>
-      <c r="S31" s="53">
+      <c r="S31" s="49">
         <v>-250</v>
       </c>
-      <c r="T31" s="53">
+      <c r="T31" s="49">
         <v>0</v>
       </c>
     </row>
@@ -3030,16 +3053,16 @@
   <dimension ref="A1:Q36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="3" width="8.54296875" style="49" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="9" style="49" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.54296875" style="49" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.26953125" style="50" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.54296875" style="51" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.54296875" style="49" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" style="49" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.54296875" style="49" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.81640625" style="49" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.453125" style="52" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="8.54296875" style="45" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="9" style="45" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.54296875" style="45" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.26953125" style="46" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.54296875" style="47" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.54296875" style="45" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" style="45" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.54296875" style="45" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.81640625" style="45" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.453125" style="48" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="1" customFormat="1" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -3299,7 +3322,7 @@
       </c>
       <c r="Q5" s="5"/>
     </row>
-    <row r="6" spans="1:17" s="1" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" s="62" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="25">
         <v>60</v>
       </c>
@@ -3309,36 +3332,36 @@
       <c r="C6" s="26">
         <v>0</v>
       </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="28">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J6" s="8">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K6" s="8">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="L6" s="29"/>
-      <c r="M6" s="7">
+      <c r="D6" s="57"/>
+      <c r="E6" s="57"/>
+      <c r="F6" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
+      <c r="I6" s="58">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J6" s="59">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K6" s="59">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="L6" s="60"/>
+      <c r="M6" s="26">
         <v>1</v>
       </c>
-      <c r="N6" s="27"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="10">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="5" t="s">
+      <c r="N6" s="57"/>
+      <c r="O6" s="57"/>
+      <c r="P6" s="61">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="62" t="s">
         <v>16</v>
       </c>
     </row>
@@ -3519,7 +3542,7 @@
       <c r="H10" s="7">
         <v>320</v>
       </c>
-      <c r="I10" s="28">
+      <c r="I10" s="27">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
@@ -3658,60 +3681,60 @@
       </c>
       <c r="Q12" s="5"/>
     </row>
-    <row r="13" spans="1:17" s="1" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="30">
+    <row r="13" spans="1:17" s="62" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="28">
         <v>80</v>
       </c>
-      <c r="B13" s="31">
-        <v>0</v>
-      </c>
-      <c r="C13" s="31">
-        <v>0</v>
-      </c>
-      <c r="D13" s="31">
+      <c r="B13" s="29">
+        <v>0</v>
+      </c>
+      <c r="C13" s="29">
+        <v>0</v>
+      </c>
+      <c r="D13" s="29">
         <v>360</v>
       </c>
-      <c r="E13" s="31">
+      <c r="E13" s="29">
         <v>364</v>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="29">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G13" s="31">
+      <c r="G13" s="29">
         <v>303</v>
       </c>
-      <c r="H13" s="32">
+      <c r="H13" s="30">
         <v>303.5</v>
       </c>
-      <c r="I13" s="33">
+      <c r="I13" s="63">
         <f t="shared" si="1"/>
         <v>0.5</v>
       </c>
-      <c r="J13" s="22">
+      <c r="J13" s="64">
         <f t="shared" si="2"/>
         <v>0.71250000000000002</v>
       </c>
-      <c r="K13" s="22">
+      <c r="K13" s="64">
         <f t="shared" si="3"/>
         <v>0.75624999999999998</v>
       </c>
-      <c r="L13" s="32">
+      <c r="L13" s="30">
         <v>0.7</v>
       </c>
-      <c r="M13" s="32">
+      <c r="M13" s="30">
         <v>0.75</v>
       </c>
-      <c r="N13" s="31">
+      <c r="N13" s="29">
         <v>-150</v>
       </c>
-      <c r="O13" s="31">
+      <c r="O13" s="29">
         <v>-160</v>
       </c>
-      <c r="P13" s="34">
+      <c r="P13" s="31">
         <v>-140</v>
       </c>
-      <c r="Q13" s="5" t="s">
+      <c r="Q13" s="62" t="s">
         <v>17</v>
       </c>
     </row>
@@ -3741,7 +3764,7 @@
       <c r="H14" s="7">
         <v>315</v>
       </c>
-      <c r="I14" s="28">
+      <c r="I14" s="27">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -3918,10 +3941,10 @@
         <f t="shared" si="3"/>
         <v>0.79</v>
       </c>
-      <c r="L17" s="35">
+      <c r="L17" s="32">
         <v>0.67</v>
       </c>
-      <c r="M17" s="35">
+      <c r="M17" s="32">
         <v>0.69</v>
       </c>
       <c r="N17" s="19">
@@ -3936,56 +3959,56 @@
       <c r="Q17" s="5"/>
     </row>
     <row r="18" spans="1:17" s="1" customFormat="1" ht="20.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="36">
+      <c r="A18" s="33">
         <v>120</v>
       </c>
-      <c r="B18" s="37">
+      <c r="B18" s="34">
         <v>90</v>
       </c>
-      <c r="C18" s="37">
-        <v>0</v>
-      </c>
-      <c r="D18" s="37">
+      <c r="C18" s="34">
+        <v>0</v>
+      </c>
+      <c r="D18" s="34">
         <v>353</v>
       </c>
-      <c r="E18" s="37">
+      <c r="E18" s="34">
         <v>356</v>
       </c>
-      <c r="F18" s="37">
+      <c r="F18" s="34">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G18" s="37">
+      <c r="G18" s="34">
         <v>304</v>
       </c>
-      <c r="H18" s="37">
+      <c r="H18" s="34">
         <v>315</v>
       </c>
-      <c r="I18" s="38">
+      <c r="I18" s="35">
         <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="J18" s="39">
+      <c r="J18" s="36">
         <f t="shared" si="2"/>
         <v>0.40833333333333333</v>
       </c>
-      <c r="K18" s="39">
+      <c r="K18" s="36">
         <f t="shared" si="3"/>
         <v>0.34166666666666667</v>
       </c>
-      <c r="L18" s="40">
+      <c r="L18" s="37">
         <v>0.77</v>
       </c>
-      <c r="M18" s="37">
+      <c r="M18" s="34">
         <v>1</v>
       </c>
-      <c r="N18" s="37">
+      <c r="N18" s="34">
         <v>-100</v>
       </c>
-      <c r="O18" s="37">
+      <c r="O18" s="34">
         <v>-130</v>
       </c>
-      <c r="P18" s="41">
+      <c r="P18" s="38">
         <v>0</v>
       </c>
       <c r="Q18" s="5"/>
@@ -4101,42 +4124,42 @@
       <c r="Q20" s="5"/>
     </row>
     <row r="21" spans="1:17" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="42">
+      <c r="A21" s="39">
         <v>120</v>
       </c>
-      <c r="B21" s="43">
-        <v>0</v>
-      </c>
-      <c r="C21" s="43">
+      <c r="B21" s="40">
+        <v>0</v>
+      </c>
+      <c r="C21" s="40">
         <v>0</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
-      <c r="F21" s="43">
+      <c r="F21" s="40">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="44">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J21" s="45">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K21" s="45">
+      <c r="I21" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="42">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K21" s="42">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L21" s="4"/>
-      <c r="M21" s="43">
+      <c r="M21" s="40">
         <v>1</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
-      <c r="P21" s="46">
+      <c r="P21" s="43">
         <v>0</v>
       </c>
       <c r="Q21" s="5"/>
@@ -4167,7 +4190,7 @@
       <c r="H22" s="9">
         <v>305.5</v>
       </c>
-      <c r="I22" s="28">
+      <c r="I22" s="27">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -4289,10 +4312,10 @@
         <f t="shared" si="3"/>
         <v>1.2</v>
       </c>
-      <c r="L24" s="35">
+      <c r="L24" s="32">
         <v>0.55000000000000004</v>
       </c>
-      <c r="M24" s="35">
+      <c r="M24" s="32">
         <v>0.6</v>
       </c>
       <c r="N24" s="19">
@@ -4332,7 +4355,7 @@
       <c r="H25" s="9">
         <v>307.5</v>
       </c>
-      <c r="I25" s="28">
+      <c r="I25" s="27">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
@@ -4454,10 +4477,10 @@
         <f t="shared" si="3"/>
         <v>0.58333333333333337</v>
       </c>
-      <c r="L27" s="35">
+      <c r="L27" s="32">
         <v>0.68</v>
       </c>
-      <c r="M27" s="35">
+      <c r="M27" s="32">
         <v>0.78</v>
       </c>
       <c r="N27" s="19">
@@ -4471,46 +4494,46 @@
       </c>
       <c r="Q27" s="5"/>
     </row>
-    <row r="28" spans="1:17" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="6">
+    <row r="28" spans="1:17" s="66" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="25">
         <v>80</v>
       </c>
-      <c r="B28" s="7">
+      <c r="B28" s="26">
         <v>90</v>
       </c>
-      <c r="C28" s="7">
+      <c r="C28" s="26">
         <v>90</v>
       </c>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="7">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="28">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J28" s="8">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K28" s="8">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="L28" s="29"/>
-      <c r="M28" s="7">
+      <c r="D28" s="57"/>
+      <c r="E28" s="57"/>
+      <c r="F28" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G28" s="57"/>
+      <c r="H28" s="57"/>
+      <c r="I28" s="58">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J28" s="59">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K28" s="59">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="L28" s="60"/>
+      <c r="M28" s="26">
         <v>1</v>
       </c>
-      <c r="N28" s="27"/>
-      <c r="O28" s="27"/>
-      <c r="P28" s="10">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="47" t="s">
+      <c r="N28" s="57"/>
+      <c r="O28" s="57"/>
+      <c r="P28" s="61">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="65" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4607,10 +4630,10 @@
         <f t="shared" si="3"/>
         <v>0.35</v>
       </c>
-      <c r="L30" s="35">
+      <c r="L30" s="32">
         <v>0.46</v>
       </c>
-      <c r="M30" s="35">
+      <c r="M30" s="32">
         <v>0.92</v>
       </c>
       <c r="N30" s="19">
@@ -4625,56 +4648,56 @@
       <c r="Q30" s="5"/>
     </row>
     <row r="31" spans="1:17" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="37">
+      <c r="A31" s="34">
         <v>100</v>
       </c>
-      <c r="B31" s="37">
+      <c r="B31" s="34">
         <v>90</v>
       </c>
-      <c r="C31" s="37">
+      <c r="C31" s="34">
         <v>90</v>
       </c>
-      <c r="D31" s="37">
+      <c r="D31" s="34">
         <v>352</v>
       </c>
-      <c r="E31" s="37">
+      <c r="E31" s="34">
         <v>374</v>
       </c>
-      <c r="F31" s="37">
+      <c r="F31" s="34">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="G31" s="37">
+      <c r="G31" s="34">
         <v>306</v>
       </c>
-      <c r="H31" s="37">
+      <c r="H31" s="34">
         <v>308</v>
       </c>
-      <c r="I31" s="38">
+      <c r="I31" s="35">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="J31" s="39">
+      <c r="J31" s="36">
         <f t="shared" si="2"/>
         <v>0.46</v>
       </c>
-      <c r="K31" s="39">
+      <c r="K31" s="36">
         <f t="shared" si="3"/>
         <v>0.66</v>
       </c>
-      <c r="L31" s="40">
+      <c r="L31" s="37">
         <v>0.55000000000000004</v>
       </c>
-      <c r="M31" s="37">
+      <c r="M31" s="34">
         <v>1</v>
       </c>
-      <c r="N31" s="37">
+      <c r="N31" s="34">
         <v>-150</v>
       </c>
-      <c r="O31" s="37">
+      <c r="O31" s="34">
         <v>-170</v>
       </c>
-      <c r="P31" s="37">
+      <c r="P31" s="34">
         <v>0</v>
       </c>
       <c r="Q31" s="5"/>
@@ -4735,56 +4758,56 @@
       <c r="Q32" s="5"/>
     </row>
     <row r="33" spans="1:17" s="1" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="43">
+      <c r="A33" s="40">
         <v>100</v>
       </c>
-      <c r="B33" s="43">
+      <c r="B33" s="40">
         <v>90</v>
       </c>
-      <c r="C33" s="43">
+      <c r="C33" s="40">
         <v>30</v>
       </c>
-      <c r="D33" s="43">
+      <c r="D33" s="40">
         <v>346</v>
       </c>
-      <c r="E33" s="43">
+      <c r="E33" s="40">
         <v>355</v>
       </c>
-      <c r="F33" s="43">
+      <c r="F33" s="40">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="G33" s="43">
+      <c r="G33" s="40">
         <v>306</v>
       </c>
-      <c r="H33" s="43">
+      <c r="H33" s="40">
         <v>329</v>
       </c>
-      <c r="I33" s="44">
+      <c r="I33" s="41">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="J33" s="45">
+      <c r="J33" s="42">
         <f t="shared" si="2"/>
         <v>0.4</v>
       </c>
-      <c r="K33" s="45">
+      <c r="K33" s="42">
         <f t="shared" si="3"/>
         <v>0.26</v>
       </c>
-      <c r="L33" s="48">
+      <c r="L33" s="44">
         <v>0.6</v>
       </c>
-      <c r="M33" s="43">
+      <c r="M33" s="40">
         <v>1</v>
       </c>
-      <c r="N33" s="43">
+      <c r="N33" s="40">
         <v>-150</v>
       </c>
-      <c r="O33" s="43">
+      <c r="O33" s="40">
         <v>-210</v>
       </c>
-      <c r="P33" s="43">
+      <c r="P33" s="40">
         <v>0</v>
       </c>
       <c r="Q33" s="5"/>
@@ -4815,7 +4838,7 @@
       <c r="H34" s="7">
         <v>314</v>
       </c>
-      <c r="I34" s="28">
+      <c r="I34" s="27">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -4937,7 +4960,7 @@
         <f t="shared" si="3"/>
         <v>0.23333333333333334</v>
       </c>
-      <c r="L36" s="35">
+      <c r="L36" s="32">
         <v>0.52</v>
       </c>
       <c r="M36" s="19">
@@ -4956,5 +4979,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>